<commit_message>
fix: make video strategy ledgers prompt-first
</commit_message>
<xml_diff>
--- a/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
+++ b/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="1" r:id="R03a65eeacd3a40dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景矩阵" sheetId="2" r:id="Rf6cb7b1d92564748"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R91161ea131c74ad0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R95634e7e9c0e4086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="R3a7329ea97dc44e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R0bb72d877d414025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R67ad511213654a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R88f0efeaaca34478"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,43 +180,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVSceneMatrix" displayName="TVSceneMatrix" ref="A3:T6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="20">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVVideoStrategy" displayName="TVVideoStrategy" ref="A3:AA6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="27">
     <x:tableColumn id="1" name="案例ID"/>
     <x:tableColumn id="2" name="案例名称"/>
-    <x:tableColumn id="3" name="唯一组合指纹"/>
-    <x:tableColumn id="4" name="物体种类"/>
-    <x:tableColumn id="5" name="物体形态"/>
-    <x:tableColumn id="6" name="环境场景"/>
-    <x:tableColumn id="7" name="覆盖状态"/>
-    <x:tableColumn id="8" name="镜头景别"/>
-    <x:tableColumn id="9" name="镜头运动"/>
-    <x:tableColumn id="10" name="人物/施工状态"/>
-    <x:tableColumn id="11" name="首帧状态"/>
-    <x:tableColumn id="12" name="视频状态"/>
-    <x:tableColumn id="13" name="图片哈希"/>
-    <x:tableColumn id="14" name="视频哈希"/>
-    <x:tableColumn id="15" name="图片模型"/>
-    <x:tableColumn id="16" name="视频模型"/>
-    <x:tableColumn id="17" name="预计视频费用（元）"/>
-    <x:tableColumn id="18" name="生成秒数"/>
-    <x:tableColumn id="19" name="任务状态"/>
-    <x:tableColumn id="20" name="项目相对路径"/>
+    <x:tableColumn id="3" name="物体种类"/>
+    <x:tableColumn id="4" name="物体形态"/>
+    <x:tableColumn id="5" name="环境场景"/>
+    <x:tableColumn id="6" name="覆盖状态"/>
+    <x:tableColumn id="7" name="镜头景别"/>
+    <x:tableColumn id="8" name="镜头运动"/>
+    <x:tableColumn id="9" name="人物/施工状态"/>
+    <x:tableColumn id="10" name="完整文生视频提示词"/>
+    <x:tableColumn id="11" name="图生视频提示词"/>
+    <x:tableColumn id="12" name="首帧提示词"/>
+    <x:tableColumn id="13" name="负面提示词"/>
+    <x:tableColumn id="14" name="唯一组合指纹"/>
+    <x:tableColumn id="15" name="首帧状态"/>
+    <x:tableColumn id="16" name="视频状态"/>
+    <x:tableColumn id="17" name="图片哈希"/>
+    <x:tableColumn id="18" name="视频哈希"/>
+    <x:tableColumn id="19" name="图片模型"/>
+    <x:tableColumn id="20" name="视频模型"/>
+    <x:tableColumn id="21" name="预计视频费用（元）"/>
+    <x:tableColumn id="22" name="生成秒数"/>
+    <x:tableColumn id="23" name="任务状态"/>
+    <x:tableColumn id="24" name="参考图片"/>
+    <x:tableColumn id="25" name="项目相对路径"/>
+    <x:tableColumn id="26" name="文生视频提示词哈希"/>
+    <x:tableColumn id="27" name="图生视频提示词哈希"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="7">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:H6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="案例ID"/>
-    <x:tableColumn id="2" name="首帧提示词"/>
-    <x:tableColumn id="3" name="视频提示词"/>
-    <x:tableColumn id="4" name="负面提示词"/>
-    <x:tableColumn id="5" name="参考图片"/>
-    <x:tableColumn id="6" name="首帧提示词哈希"/>
-    <x:tableColumn id="7" name="视频提示词哈希"/>
+    <x:tableColumn id="2" name="完整文生视频提示词"/>
+    <x:tableColumn id="3" name="图生视频提示词"/>
+    <x:tableColumn id="4" name="首帧提示词"/>
+    <x:tableColumn id="5" name="负面提示词"/>
+    <x:tableColumn id="6" name="参考图片"/>
+    <x:tableColumn id="7" name="文生视频提示词哈希"/>
+    <x:tableColumn id="8" name="图生视频提示词哈希"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -429,6 +437,470 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="70" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="70" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="70" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="70" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="38" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="L1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="M1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="N1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="O1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="P1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="Q1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="R1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="S1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="T1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="U1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="V1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="W1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="X1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="Y1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="Z1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+      <x:c r="AA1" s="3" t="str">
+        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="10" t="str">
+        <x:v>案例ID</x:v>
+      </x:c>
+      <x:c r="B3" s="15" t="str">
+        <x:v>案例名称</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="str">
+        <x:v>物体种类</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="str">
+        <x:v>物体形态</x:v>
+      </x:c>
+      <x:c r="E3" s="15" t="str">
+        <x:v>环境场景</x:v>
+      </x:c>
+      <x:c r="F3" s="15" t="str">
+        <x:v>覆盖状态</x:v>
+      </x:c>
+      <x:c r="G3" s="15" t="str">
+        <x:v>镜头景别</x:v>
+      </x:c>
+      <x:c r="H3" s="15" t="str">
+        <x:v>镜头运动</x:v>
+      </x:c>
+      <x:c r="I3" s="15" t="str">
+        <x:v>人物/施工状态</x:v>
+      </x:c>
+      <x:c r="J3" s="15" t="str">
+        <x:v>完整文生视频提示词</x:v>
+      </x:c>
+      <x:c r="K3" s="15" t="str">
+        <x:v>图生视频提示词</x:v>
+      </x:c>
+      <x:c r="L3" s="15" t="str">
+        <x:v>首帧提示词</x:v>
+      </x:c>
+      <x:c r="M3" s="15" t="str">
+        <x:v>负面提示词</x:v>
+      </x:c>
+      <x:c r="N3" s="15" t="str">
+        <x:v>唯一组合指纹</x:v>
+      </x:c>
+      <x:c r="O3" s="15" t="str">
+        <x:v>首帧状态</x:v>
+      </x:c>
+      <x:c r="P3" s="15" t="str">
+        <x:v>视频状态</x:v>
+      </x:c>
+      <x:c r="Q3" s="15" t="str">
+        <x:v>图片哈希</x:v>
+      </x:c>
+      <x:c r="R3" s="15" t="str">
+        <x:v>视频哈希</x:v>
+      </x:c>
+      <x:c r="S3" s="15" t="str">
+        <x:v>图片模型</x:v>
+      </x:c>
+      <x:c r="T3" s="15" t="str">
+        <x:v>视频模型</x:v>
+      </x:c>
+      <x:c r="U3" s="15" t="str">
+        <x:v>预计视频费用（元）</x:v>
+      </x:c>
+      <x:c r="V3" s="15" t="str">
+        <x:v>生成秒数</x:v>
+      </x:c>
+      <x:c r="W3" s="15" t="str">
+        <x:v>任务状态</x:v>
+      </x:c>
+      <x:c r="X3" s="15" t="str">
+        <x:v>参考图片</x:v>
+      </x:c>
+      <x:c r="Y3" s="15" t="str">
+        <x:v>项目相对路径</x:v>
+      </x:c>
+      <x:c r="Z3" s="15" t="str">
+        <x:v>文生视频提示词哈希</x:v>
+      </x:c>
+      <x:c r="AA3" s="11" t="str">
+        <x:v>图生视频提示词哈希</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="300" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>v01-s01</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>电视案例01</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>television</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>65-inch ultra-thin wall-mounted flat panel</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>bright Scandinavian living room under repainting</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>fully covered by a taut rectangular clear film curtain</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>wide full-wall shot</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>slow left-to-right lateral slider</x:v>
+      </x:c>
+      <x:c r="I4" s="16" t="str">
+        <x:v>no person; completed protection state</x:v>
+      </x:c>
+      <x:c r="J4" s="16" t="str">
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 65-inch ultra-thin wall-mounted flat panel. Environment: bright Scandinavian living room under repainting. Coverage state: fully covered by a taut rectangular clear film curtain. Shot scale: wide full-wall shot. Camera motion: slow left-to-right lateral slider. Person or work state: no person; completed protection state. Opening visual and product geometry: Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="K4" s="16" t="str">
+        <x:v>Maintain the approved Scandinavian living-room keyframe and exact integrated product geometry. The 65-inch television stays fully behind one continuous clear film sheet; the yellow wall tape stays bonded across the complete film top edge with aligned endpoints. Execute a slow left-to-right lateral slider move that reveals mild parallax between the oak console and pale wall. Only tiny natural surface shimmer may occur in the film; no tear, opening, doubled flap, loose tape, uncovered television, person, installation action, transformation, flicker, text or logo.</x:v>
+      </x:c>
+      <x:c r="L4" s="16" t="str">
+        <x:v>Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="M4" s="16" t="str">
+        <x:v>broken film, split plastic, extra tape, exposed screen, tape on television, duplicate sheet</x:v>
+      </x:c>
+      <x:c r="N4" s="16" t="str">
+        <x:v>25a85bb6a5e1</x:v>
+      </x:c>
+      <x:c r="O4" s="16" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P4" s="16" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="Q4" s="16" t="str">
+        <x:v>5a1fe65799bc295023a3214271fca0dc2e937204ba29e1fb377d2f1808602caf</x:v>
+      </x:c>
+      <x:c r="R4" s="16" t="str">
+        <x:v>e1cbb570af138da14ef24c8185c9ded84e2c9005570140ac3b2f8a9d6961889b</x:v>
+      </x:c>
+      <x:c r="S4" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="T4" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="U4" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="V4" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W4" s="16" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="X4" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
+      <x:c r="Y4" s="16" t="str">
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
+      </x:c>
+      <x:c r="Z4" s="16" t="str">
+        <x:v>a432a56c0d26223d</x:v>
+      </x:c>
+      <x:c r="AA4" s="16" t="str">
+        <x:v>989be0d00589988c</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="300" customHeight="1">
+      <x:c r="A5" s="16" t="str">
+        <x:v>v02-s01</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="str">
+        <x:v>电视案例02</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="str">
+        <x:v>television</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
+        <x:v>43-inch compact wall-mounted flat panel</x:v>
+      </x:c>
+      <x:c r="E5" s="16" t="str">
+        <x:v>warm boutique-hotel bedroom renovation</x:v>
+      </x:c>
+      <x:c r="F5" s="16" t="str">
+        <x:v>fully covered with softly draped side and lower margins</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="str">
+        <x:v>three-quarter medium shot from the right</x:v>
+      </x:c>
+      <x:c r="H5" s="16" t="str">
+        <x:v>slow rightward dolly with restrained parallax</x:v>
+      </x:c>
+      <x:c r="I5" s="16" t="str">
+        <x:v>professional painter kneeling at frame left and visually inspecting without touching</x:v>
+      </x:c>
+      <x:c r="J5" s="16" t="str">
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 43-inch compact wall-mounted flat panel. Environment: warm boutique-hotel bedroom renovation. Coverage state: fully covered with softly draped side and lower margins. Shot scale: three-quarter medium shot from the right. Camera motion: slow rightward dolly with restrained parallax. Person or work state: professional painter kneeling at frame left and visually inspecting without touching. Opening visual and product geometry: Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="K5" s="16" t="str">
+        <x:v>Preserve the boutique-hotel bedroom, compact television, kneeling painter and the approved one-piece tape-film structure. Move the camera slowly to the right for restrained parallax across the walnut desk. The painter only shifts his gaze from the lower film margin to the yellow tape and gives one small satisfied nod; he never touches the product. The transparent sheet remains one intact layer covering the complete television, and both film edges remain aligned with the tape endpoints. No tear, flap, second layer, tape movement, installation, exposed screen, body occlusion, lip movement, text or logo.</x:v>
+      </x:c>
+      <x:c r="L5" s="16" t="str">
+        <x:v>Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="M5" s="16" t="str">
+        <x:v>hands touching film, torn plastic, extra tape, person blocking product, exposed television</x:v>
+      </x:c>
+      <x:c r="N5" s="16" t="str">
+        <x:v>09c0a89c716c</x:v>
+      </x:c>
+      <x:c r="O5" s="16" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P5" s="16" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="Q5" s="16" t="str">
+        <x:v>0303b24d530d619f3aed59ac14065486768a84e9a52c98a21a4b053bd4db78bc</x:v>
+      </x:c>
+      <x:c r="R5" s="16" t="str">
+        <x:v>c3db73e0a1871d0c6ec6e6918d7d6b3fef82e941b093320cfe58808bea9c58b7</x:v>
+      </x:c>
+      <x:c r="S5" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="T5" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="U5" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="V5" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W5" s="16" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="X5" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
+      <x:c r="Y5" s="16" t="str">
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
+      </x:c>
+      <x:c r="Z5" s="16" t="str">
+        <x:v>c6ef5a34bdd7a12b</x:v>
+      </x:c>
+      <x:c r="AA5" s="16" t="str">
+        <x:v>3d95e6b36115d38a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="300" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>v03-s01</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>电视案例03</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="str">
+        <x:v>television</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>75-inch wide wall-mounted flat panel</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>industrial loft media room with smooth white mounting panel</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>fully covered with broad transparent margins and lightly tensioned lower edge</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>low-angle wide shot</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
+        <x:v>gentle upward tilt from console to tape line</x:v>
+      </x:c>
+      <x:c r="I6" s="16" t="str">
+        <x:v>standing painter at far right pointing beside the protected area</x:v>
+      </x:c>
+      <x:c r="J6" s="16" t="str">
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 75-inch wide wall-mounted flat panel. Environment: industrial loft media room with smooth white mounting panel. Coverage state: fully covered with broad transparent margins and lightly tensioned lower edge. Shot scale: low-angle wide shot. Camera motion: gentle upward tilt from console to tape line. Person or work state: standing painter at far right pointing beside the protected area. Opening visual and product geometry: Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="str">
+        <x:v>Keep the industrial loft, 75-inch television, standing painter and full-width one-piece film installation unchanged. Begin low on the black metal console and perform a gentle upward camera tilt ending on the straight yellow tape line. The painter makes one restrained open-palm presentation gesture beside the film boundary without touching it. Throughout the tilt the television remains fully behind one continuous transparent sheet with broad margins; tape and film endpoints stay aligned. No split, hole, double flap, extra tape, exposed bezel, strong wind, installation, speech, text or logo.</x:v>
+      </x:c>
+      <x:c r="L6" s="16" t="str">
+        <x:v>Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="M6" s="16" t="str">
+        <x:v>camera orbit, broken film, tape overhang, presenter blocking television, extra plastic layer</x:v>
+      </x:c>
+      <x:c r="N6" s="16" t="str">
+        <x:v>b3b654812d2d</x:v>
+      </x:c>
+      <x:c r="O6" s="16" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P6" s="16" t="str">
+        <x:v>淘汰</x:v>
+      </x:c>
+      <x:c r="Q6" s="16" t="str">
+        <x:v>9fbc6f466b567258e7d6339a36bc6db7522e8b1c60a3d3e55c006dd0606b9060</x:v>
+      </x:c>
+      <x:c r="R6" s="16" t="str">
+        <x:v>93ae4e3521b49c08de0e3073cdcfb5313fe8e52aabcf823bb6722e7fcd8bb870</x:v>
+      </x:c>
+      <x:c r="S6" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="T6" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="U6" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="V6" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W6" s="16" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="X6" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
+      <x:c r="Y6" s="16" t="str">
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
+      </x:c>
+      <x:c r="Z6" s="16" t="str">
+        <x:v>220888f5910eebd3</x:v>
+      </x:c>
+      <x:c r="AA6" s="16" t="str">
+        <x:v>159e41806fbf71f6</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:AA1"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="O4:P6">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="通过"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="待"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f8ee893e244c3e"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
@@ -482,7 +954,7 @@
         <x:v>差异化案例数</x:v>
       </x:c>
       <x:c r="B4" s="17" t="n">
-        <x:f>COUNTA('场景矩阵'!$A$4:$A$100)</x:f>
+        <x:f>COUNTA('视频策略库'!$A$4:$A$100)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C4" s="17"/>
@@ -495,7 +967,7 @@
         <x:v>唯一七维组合数</x:v>
       </x:c>
       <x:c r="B5" s="17" t="n">
-        <x:f>COUNTA('场景矩阵'!$C$4:$C$100)</x:f>
+        <x:f>COUNTA('视频策略库'!$N$4:$N$100)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
@@ -508,7 +980,7 @@
         <x:v>首帧通过数</x:v>
       </x:c>
       <x:c r="B6" s="17" t="n">
-        <x:f>COUNTIF('场景矩阵'!$K$4:$K$100,"通过")</x:f>
+        <x:f>COUNTIF('视频策略库'!$O$4:$O$100,"通过")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
@@ -521,7 +993,7 @@
         <x:v>视频通过数</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
-        <x:f>COUNTIF('场景矩阵'!$L$4:$L$100,"通过")</x:f>
+        <x:f>COUNTIF('视频策略库'!$P$4:$P$100,"通过")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
@@ -534,7 +1006,7 @@
         <x:v>预计视频费用（元）</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:f>ROUND(SUM('场景矩阵'!$Q$4:$Q$100),2)</x:f>
+        <x:f>ROUND(SUM('视频策略库'!$U$4:$U$100),2)</x:f>
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
@@ -577,7 +1049,7 @@
         <x:v>台账定位</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>用于筛选策略、查看提示词、追踪验收与复盘淘汰素材</x:v>
+        <x:v>主表逐行列出七维组合及其完整文生视频提示词；统计页仅用于辅助查看</x:v>
       </x:c>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="19"/>
@@ -608,392 +1080,44 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="34" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="L1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="M1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="N1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="O1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="P1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="Q1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="R1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="S1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-      <x:c r="T1" s="3" t="str">
-        <x:v>电视场景矩阵｜七维组合与生产状态</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" s="10" t="str">
-        <x:v>案例ID</x:v>
-      </x:c>
-      <x:c r="B3" s="15" t="str">
-        <x:v>案例名称</x:v>
-      </x:c>
-      <x:c r="C3" s="15" t="str">
-        <x:v>唯一组合指纹</x:v>
-      </x:c>
-      <x:c r="D3" s="15" t="str">
-        <x:v>物体种类</x:v>
-      </x:c>
-      <x:c r="E3" s="15" t="str">
-        <x:v>物体形态</x:v>
-      </x:c>
-      <x:c r="F3" s="15" t="str">
-        <x:v>环境场景</x:v>
-      </x:c>
-      <x:c r="G3" s="15" t="str">
-        <x:v>覆盖状态</x:v>
-      </x:c>
-      <x:c r="H3" s="15" t="str">
-        <x:v>镜头景别</x:v>
-      </x:c>
-      <x:c r="I3" s="15" t="str">
-        <x:v>镜头运动</x:v>
-      </x:c>
-      <x:c r="J3" s="15" t="str">
-        <x:v>人物/施工状态</x:v>
-      </x:c>
-      <x:c r="K3" s="15" t="str">
-        <x:v>首帧状态</x:v>
-      </x:c>
-      <x:c r="L3" s="15" t="str">
-        <x:v>视频状态</x:v>
-      </x:c>
-      <x:c r="M3" s="15" t="str">
-        <x:v>图片哈希</x:v>
-      </x:c>
-      <x:c r="N3" s="15" t="str">
-        <x:v>视频哈希</x:v>
-      </x:c>
-      <x:c r="O3" s="15" t="str">
-        <x:v>图片模型</x:v>
-      </x:c>
-      <x:c r="P3" s="15" t="str">
-        <x:v>视频模型</x:v>
-      </x:c>
-      <x:c r="Q3" s="15" t="str">
-        <x:v>预计视频费用（元）</x:v>
-      </x:c>
-      <x:c r="R3" s="15" t="str">
-        <x:v>生成秒数</x:v>
-      </x:c>
-      <x:c r="S3" s="15" t="str">
-        <x:v>任务状态</x:v>
-      </x:c>
-      <x:c r="T3" s="11" t="str">
-        <x:v>项目相对路径</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="16" t="str">
-        <x:v>v01-s01</x:v>
-      </x:c>
-      <x:c r="B4" s="16" t="str">
-        <x:v>电视案例01</x:v>
-      </x:c>
-      <x:c r="C4" s="16" t="str">
-        <x:v>25a85bb6a5e1</x:v>
-      </x:c>
-      <x:c r="D4" s="16" t="str">
-        <x:v>television</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>65-inch ultra-thin wall-mounted flat panel</x:v>
-      </x:c>
-      <x:c r="F4" s="16" t="str">
-        <x:v>bright Scandinavian living room under repainting</x:v>
-      </x:c>
-      <x:c r="G4" s="16" t="str">
-        <x:v>fully covered by a taut rectangular clear film curtain</x:v>
-      </x:c>
-      <x:c r="H4" s="16" t="str">
-        <x:v>wide full-wall shot</x:v>
-      </x:c>
-      <x:c r="I4" s="16" t="str">
-        <x:v>slow left-to-right lateral slider</x:v>
-      </x:c>
-      <x:c r="J4" s="16" t="str">
-        <x:v>no person; completed protection state</x:v>
-      </x:c>
-      <x:c r="K4" s="16" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="L4" s="16" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="M4" s="16" t="str">
-        <x:v>5a1fe65799bc295023a3214271fca0dc2e937204ba29e1fb377d2f1808602caf</x:v>
-      </x:c>
-      <x:c r="N4" s="16" t="str">
-        <x:v>e1cbb570af138da14ef24c8185c9ded84e2c9005570140ac3b2f8a9d6961889b</x:v>
-      </x:c>
-      <x:c r="O4" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="P4" s="16" t="str">
-        <x:v>grok-imagine-video-1.5-fast</x:v>
-      </x:c>
-      <x:c r="Q4" s="20" t="n">
-        <x:v>0.6</x:v>
-      </x:c>
-      <x:c r="R4" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="S4" s="16" t="str">
-        <x:v>completed</x:v>
-      </x:c>
-      <x:c r="T4" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="16" t="str">
-        <x:v>v02-s01</x:v>
-      </x:c>
-      <x:c r="B5" s="16" t="str">
-        <x:v>电视案例02</x:v>
-      </x:c>
-      <x:c r="C5" s="16" t="str">
-        <x:v>09c0a89c716c</x:v>
-      </x:c>
-      <x:c r="D5" s="16" t="str">
-        <x:v>television</x:v>
-      </x:c>
-      <x:c r="E5" s="16" t="str">
-        <x:v>43-inch compact wall-mounted flat panel</x:v>
-      </x:c>
-      <x:c r="F5" s="16" t="str">
-        <x:v>warm boutique-hotel bedroom renovation</x:v>
-      </x:c>
-      <x:c r="G5" s="16" t="str">
-        <x:v>fully covered with softly draped side and lower margins</x:v>
-      </x:c>
-      <x:c r="H5" s="16" t="str">
-        <x:v>three-quarter medium shot from the right</x:v>
-      </x:c>
-      <x:c r="I5" s="16" t="str">
-        <x:v>slow rightward dolly with restrained parallax</x:v>
-      </x:c>
-      <x:c r="J5" s="16" t="str">
-        <x:v>professional painter kneeling at frame left and visually inspecting without touching</x:v>
-      </x:c>
-      <x:c r="K5" s="16" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="L5" s="16" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="M5" s="16" t="str">
-        <x:v>0303b24d530d619f3aed59ac14065486768a84e9a52c98a21a4b053bd4db78bc</x:v>
-      </x:c>
-      <x:c r="N5" s="16" t="str">
-        <x:v>c3db73e0a1871d0c6ec6e6918d7d6b3fef82e941b093320cfe58808bea9c58b7</x:v>
-      </x:c>
-      <x:c r="O5" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="P5" s="16" t="str">
-        <x:v>grok-imagine-video-1.5-fast</x:v>
-      </x:c>
-      <x:c r="Q5" s="20" t="n">
-        <x:v>0.6</x:v>
-      </x:c>
-      <x:c r="R5" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="S5" s="16" t="str">
-        <x:v>completed</x:v>
-      </x:c>
-      <x:c r="T5" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="16" t="str">
-        <x:v>v03-s01</x:v>
-      </x:c>
-      <x:c r="B6" s="16" t="str">
-        <x:v>电视案例03</x:v>
-      </x:c>
-      <x:c r="C6" s="16" t="str">
-        <x:v>b3b654812d2d</x:v>
-      </x:c>
-      <x:c r="D6" s="16" t="str">
-        <x:v>television</x:v>
-      </x:c>
-      <x:c r="E6" s="16" t="str">
-        <x:v>75-inch wide wall-mounted flat panel</x:v>
-      </x:c>
-      <x:c r="F6" s="16" t="str">
-        <x:v>industrial loft media room with smooth white mounting panel</x:v>
-      </x:c>
-      <x:c r="G6" s="16" t="str">
-        <x:v>fully covered with broad transparent margins and lightly tensioned lower edge</x:v>
-      </x:c>
-      <x:c r="H6" s="16" t="str">
-        <x:v>low-angle wide shot</x:v>
-      </x:c>
-      <x:c r="I6" s="16" t="str">
-        <x:v>gentle upward tilt from console to tape line</x:v>
-      </x:c>
-      <x:c r="J6" s="16" t="str">
-        <x:v>standing painter at far right pointing beside the protected area</x:v>
-      </x:c>
-      <x:c r="K6" s="16" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="L6" s="16" t="str">
-        <x:v>淘汰</x:v>
-      </x:c>
-      <x:c r="M6" s="16" t="str">
-        <x:v>9fbc6f466b567258e7d6339a36bc6db7522e8b1c60a3d3e55c006dd0606b9060</x:v>
-      </x:c>
-      <x:c r="N6" s="16" t="str">
-        <x:v>93ae4e3521b49c08de0e3073cdcfb5313fe8e52aabcf823bb6722e7fcd8bb870</x:v>
-      </x:c>
-      <x:c r="O6" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="P6" s="16" t="str">
-        <x:v>grok-imagine-video-1.5-fast</x:v>
-      </x:c>
-      <x:c r="Q6" s="20" t="n">
-        <x:v>0.6</x:v>
-      </x:c>
-      <x:c r="R6" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="S6" s="16" t="str">
-        <x:v>completed</x:v>
-      </x:c>
-      <x:c r="T6" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:T1"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="K4:L6">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="通过"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="淘汰"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="待"/>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cd4fd9f247a44b7"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="70" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>电视提示词档案｜一条提示词对应一条视频</x:v>
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -1001,100 +1125,112 @@
         <x:v>案例ID</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
+        <x:v>完整文生视频提示词</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="str">
+        <x:v>图生视频提示词</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="str">
         <x:v>首帧提示词</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="str">
-        <x:v>视频提示词</x:v>
-      </x:c>
-      <x:c r="D3" s="15" t="str">
+      <x:c r="E3" s="15" t="str">
         <x:v>负面提示词</x:v>
       </x:c>
-      <x:c r="E3" s="15" t="str">
+      <x:c r="F3" s="15" t="str">
         <x:v>参考图片</x:v>
       </x:c>
-      <x:c r="F3" s="15" t="str">
-        <x:v>首帧提示词哈希</x:v>
-      </x:c>
-      <x:c r="G3" s="11" t="str">
-        <x:v>视频提示词哈希</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="132" customHeight="1">
+      <x:c r="G3" s="15" t="str">
+        <x:v>文生视频提示词哈希</x:v>
+      </x:c>
+      <x:c r="H3" s="11" t="str">
+        <x:v>图生视频提示词哈希</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="300" customHeight="1">
       <x:c r="A4" s="16" t="str">
         <x:v>v01-s01</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark.</x:v>
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 65-inch ultra-thin wall-mounted flat panel. Environment: bright Scandinavian living room under repainting. Coverage state: fully covered by a taut rectangular clear film curtain. Shot scale: wide full-wall shot. Camera motion: slow left-to-right lateral slider. Person or work state: no person; completed protection state. Opening visual and product geometry: Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
         <x:v>Maintain the approved Scandinavian living-room keyframe and exact integrated product geometry. The 65-inch television stays fully behind one continuous clear film sheet; the yellow wall tape stays bonded across the complete film top edge with aligned endpoints. Execute a slow left-to-right lateral slider move that reveals mild parallax between the oak console and pale wall. Only tiny natural surface shimmer may occur in the film; no tear, opening, doubled flap, loose tape, uncovered television, person, installation action, transformation, flicker, text or logo.</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
+        <x:v>Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
         <x:v>broken film, split plastic, extra tape, exposed screen, tape on television, duplicate sheet</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str">
+      <x:c r="F4" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="str">
-        <x:v>64ebb241c4793691</x:v>
-      </x:c>
       <x:c r="G4" s="16" t="str">
+        <x:v>a432a56c0d26223d</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
         <x:v>989be0d00589988c</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="132" customHeight="1">
+    <x:row r="5" ht="300" customHeight="1">
       <x:c r="A5" s="16" t="str">
         <x:v>v02-s01</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark.</x:v>
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 43-inch compact wall-mounted flat panel. Environment: warm boutique-hotel bedroom renovation. Coverage state: fully covered with softly draped side and lower margins. Shot scale: three-quarter medium shot from the right. Camera motion: slow rightward dolly with restrained parallax. Person or work state: professional painter kneeling at frame left and visually inspecting without touching. Opening visual and product geometry: Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
         <x:v>Preserve the boutique-hotel bedroom, compact television, kneeling painter and the approved one-piece tape-film structure. Move the camera slowly to the right for restrained parallax across the walnut desk. The painter only shifts his gaze from the lower film margin to the yellow tape and gives one small satisfied nod; he never touches the product. The transparent sheet remains one intact layer covering the complete television, and both film edges remain aligned with the tape endpoints. No tear, flap, second layer, tape movement, installation, exposed screen, body occlusion, lip movement, text or logo.</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
+        <x:v>Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="E5" s="16" t="str">
         <x:v>hands touching film, torn plastic, extra tape, person blocking product, exposed television</x:v>
       </x:c>
-      <x:c r="E5" s="16" t="str">
+      <x:c r="F5" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
-      <x:c r="F5" s="16" t="str">
-        <x:v>7d7c67b09261bc1a</x:v>
-      </x:c>
       <x:c r="G5" s="16" t="str">
+        <x:v>c6ef5a34bdd7a12b</x:v>
+      </x:c>
+      <x:c r="H5" s="16" t="str">
         <x:v>3d95e6b36115d38a</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="132" customHeight="1">
+    <x:row r="6" ht="300" customHeight="1">
       <x:c r="A6" s="16" t="str">
         <x:v>v03-s01</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark.</x:v>
+        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 75-inch wide wall-mounted flat panel. Environment: industrial loft media room with smooth white mounting panel. Coverage state: fully covered with broad transparent margins and lightly tensioned lower edge. Shot scale: low-angle wide shot. Camera motion: gentle upward tilt from console to tape line. Person or work state: standing painter at far right pointing beside the protected area. Opening visual and product geometry: Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
         <x:v>Keep the industrial loft, 75-inch television, standing painter and full-width one-piece film installation unchanged. Begin low on the black metal console and perform a gentle upward camera tilt ending on the straight yellow tape line. The painter makes one restrained open-palm presentation gesture beside the film boundary without touching it. Throughout the tilt the television remains fully behind one continuous transparent sheet with broad margins; tape and film endpoints stay aligned. No split, hole, double flap, extra tape, exposed bezel, strong wind, installation, speech, text or logo.</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
+        <x:v>Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark.</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
         <x:v>camera orbit, broken film, tape overhang, presenter blocking television, extra plastic layer</x:v>
       </x:c>
-      <x:c r="E6" s="16" t="str">
+      <x:c r="F6" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
-      <x:c r="F6" s="16" t="str">
-        <x:v>2882a5dbf4beea98</x:v>
-      </x:c>
       <x:c r="G6" s="16" t="str">
+        <x:v>220888f5910eebd3</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
         <x:v>159e41806fbf71f6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80fa75427d06448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3ef628e33604f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1199,7 +1335,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4748318de2d4dc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f34302527ad4904"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: localize video strategy ledgers
</commit_message>
<xml_diff>
--- a/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
+++ b/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="R3a7329ea97dc44e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R0bb72d877d414025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R67ad511213654a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R88f0efeaaca34478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Ra02494dbf7224a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R792018fec5f84ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R639119724e834264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="Rdb62b6ab7e824234"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -640,40 +640,40 @@
         <x:v>电视案例01</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>television</x:v>
+        <x:v>电视</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>65-inch ultra-thin wall-mounted flat panel</x:v>
+        <x:v>65英寸超薄壁挂平板电视</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
-        <x:v>bright Scandinavian living room under repainting</x:v>
+        <x:v>正在重新粉刷的明亮北欧风客厅</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
-        <x:v>fully covered by a taut rectangular clear film curtain</x:v>
+        <x:v>一整张绷紧的矩形透明膜完整覆盖电视，并在四周留出清晰边界</x:v>
       </x:c>
       <x:c r="G4" s="16" t="str">
-        <x:v>wide full-wall shot</x:v>
+        <x:v>正面墙体全景</x:v>
       </x:c>
       <x:c r="H4" s="16" t="str">
-        <x:v>slow left-to-right lateral slider</x:v>
+        <x:v>镜头从左向右缓慢横移</x:v>
       </x:c>
       <x:c r="I4" s="16" t="str">
-        <x:v>no person; completed protection state</x:v>
+        <x:v>无人物，防护施工已经完成</x:v>
       </x:c>
       <x:c r="J4" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 65-inch ultra-thin wall-mounted flat panel. Environment: bright Scandinavian living room under repainting. Coverage state: fully covered by a taut rectangular clear film curtain. Shot scale: wide full-wall shot. Camera motion: slow left-to-right lateral slider. Person or work state: no person; completed protection state. Opening visual and product geometry: Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：65英寸超薄壁挂平板电视。 环境场景：正在重新粉刷的明亮北欧风客厅。覆盖状态：一整张绷紧的矩形透明膜完整覆盖电视，并在四周留出清晰边界。 镜头景别：正面墙体全景；镜头运动：镜头从左向右缓慢横移。 人物或施工状态：无人物，防护施工已经完成。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。 动态过程：以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="K4" s="16" t="str">
-        <x:v>Maintain the approved Scandinavian living-room keyframe and exact integrated product geometry. The 65-inch television stays fully behind one continuous clear film sheet; the yellow wall tape stays bonded across the complete film top edge with aligned endpoints. Execute a slow left-to-right lateral slider move that reveals mild parallax between the oak console and pale wall. Only tiny natural surface shimmer may occur in the film; no tear, opening, doubled flap, loose tape, uncovered television, person, installation action, transformation, flicker, text or logo.</x:v>
+        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
       </x:c>
       <x:c r="L4" s="16" t="str">
-        <x:v>Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
       </x:c>
       <x:c r="M4" s="16" t="str">
-        <x:v>broken film, split plastic, extra tape, exposed screen, tape on television, duplicate sheet</x:v>
+        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
       </x:c>
       <x:c r="N4" s="16" t="str">
-        <x:v>25a85bb6a5e1</x:v>
+        <x:v>a2db2b40b93d</x:v>
       </x:c>
       <x:c r="O4" s="16" t="str">
         <x:v>通过</x:v>
@@ -700,7 +700,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="W4" s="16" t="str">
-        <x:v>completed</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="X4" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
@@ -709,10 +709,10 @@
         <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Z4" s="16" t="str">
-        <x:v>a432a56c0d26223d</x:v>
+        <x:v>4608463e01bf6f70</x:v>
       </x:c>
       <x:c r="AA4" s="16" t="str">
-        <x:v>989be0d00589988c</x:v>
+        <x:v>365df2c1d064cfcd</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="300" customHeight="1">
@@ -723,40 +723,40 @@
         <x:v>电视案例02</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>television</x:v>
+        <x:v>电视</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>43-inch compact wall-mounted flat panel</x:v>
+        <x:v>43英寸紧凑型壁挂平板电视</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>warm boutique-hotel bedroom renovation</x:v>
+        <x:v>正在翻新的暖色精品酒店客房</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>fully covered with softly draped side and lower margins</x:v>
+        <x:v>透明膜完整覆盖电视，侧边和下沿呈轻微自然垂坠</x:v>
       </x:c>
       <x:c r="G5" s="16" t="str">
-        <x:v>three-quarter medium shot from the right</x:v>
+        <x:v>从右侧拍摄的四分之三中景</x:v>
       </x:c>
       <x:c r="H5" s="16" t="str">
-        <x:v>slow rightward dolly with restrained parallax</x:v>
+        <x:v>镜头缓慢向右移动，产生克制的空间视差</x:v>
       </x:c>
       <x:c r="I5" s="16" t="str">
-        <x:v>professional painter kneeling at frame left and visually inspecting without touching</x:v>
+        <x:v>专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品</x:v>
       </x:c>
       <x:c r="J5" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 43-inch compact wall-mounted flat panel. Environment: warm boutique-hotel bedroom renovation. Coverage state: fully covered with softly draped side and lower margins. Shot scale: three-quarter medium shot from the right. Camera motion: slow rightward dolly with restrained parallax. Person or work state: professional painter kneeling at frame left and visually inspecting without touching. Opening visual and product geometry: Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：43英寸紧凑型壁挂平板电视。 环境场景：正在翻新的暖色精品酒店客房。覆盖状态：透明膜完整覆盖电视，侧边和下沿呈轻微自然垂坠。 镜头景别：从右侧拍摄的四分之三中景；镜头运动：镜头缓慢向右移动，产生克制的空间视差。 人物或施工状态：专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。 动态过程：以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="K5" s="16" t="str">
-        <x:v>Preserve the boutique-hotel bedroom, compact television, kneeling painter and the approved one-piece tape-film structure. Move the camera slowly to the right for restrained parallax across the walnut desk. The painter only shifts his gaze from the lower film margin to the yellow tape and gives one small satisfied nod; he never touches the product. The transparent sheet remains one intact layer covering the complete television, and both film edges remain aligned with the tape endpoints. No tear, flap, second layer, tape movement, installation, exposed screen, body occlusion, lip movement, text or logo.</x:v>
+        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str">
-        <x:v>Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="M5" s="16" t="str">
-        <x:v>hands touching film, torn plastic, extra tape, person blocking product, exposed television</x:v>
+        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
       </x:c>
       <x:c r="N5" s="16" t="str">
-        <x:v>09c0a89c716c</x:v>
+        <x:v>9d72917b4125</x:v>
       </x:c>
       <x:c r="O5" s="16" t="str">
         <x:v>通过</x:v>
@@ -783,7 +783,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="W5" s="16" t="str">
-        <x:v>completed</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="X5" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
@@ -792,10 +792,10 @@
         <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Z5" s="16" t="str">
-        <x:v>c6ef5a34bdd7a12b</x:v>
+        <x:v>4cb8aea4db242032</x:v>
       </x:c>
       <x:c r="AA5" s="16" t="str">
-        <x:v>3d95e6b36115d38a</x:v>
+        <x:v>8c9b3e0b2372ea58</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="300" customHeight="1">
@@ -806,40 +806,40 @@
         <x:v>电视案例03</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>television</x:v>
+        <x:v>电视</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
-        <x:v>75-inch wide wall-mounted flat panel</x:v>
+        <x:v>75英寸超宽壁挂平板电视</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>industrial loft media room with smooth white mounting panel</x:v>
+        <x:v>带白色安装墙面的工业风阁楼影音区</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>fully covered with broad transparent margins and lightly tensioned lower edge</x:v>
+        <x:v>宽幅透明膜完整覆盖电视，左右留出宽边，下沿轻微绷紧</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>low-angle wide shot</x:v>
+        <x:v>低机位广角镜头</x:v>
       </x:c>
       <x:c r="H6" s="16" t="str">
-        <x:v>gentle upward tilt from console to tape line</x:v>
+        <x:v>镜头从下方电视柜缓慢向上抬升至黄色胶带</x:v>
       </x:c>
       <x:c r="I6" s="16" t="str">
-        <x:v>standing painter at far right pointing beside the protected area</x:v>
+        <x:v>专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势</x:v>
       </x:c>
       <x:c r="J6" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 75-inch wide wall-mounted flat panel. Environment: industrial loft media room with smooth white mounting panel. Coverage state: fully covered with broad transparent margins and lightly tensioned lower edge. Shot scale: low-angle wide shot. Camera motion: gentle upward tilt from console to tape line. Person or work state: standing painter at far right pointing beside the protected area. Opening visual and product geometry: Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：75英寸超宽壁挂平板电视。 环境场景：带白色安装墙面的工业风阁楼影音区。覆盖状态：宽幅透明膜完整覆盖电视，左右留出宽边，下沿轻微绷紧。 镜头景别：低机位广角镜头；镜头运动：镜头从下方电视柜缓慢向上抬升至黄色胶带。 人物或施工状态：专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。 动态过程：以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="K6" s="16" t="str">
-        <x:v>Keep the industrial loft, 75-inch television, standing painter and full-width one-piece film installation unchanged. Begin low on the black metal console and perform a gentle upward camera tilt ending on the straight yellow tape line. The painter makes one restrained open-palm presentation gesture beside the film boundary without touching it. Throughout the tilt the television remains fully behind one continuous transparent sheet with broad margins; tape and film endpoints stay aligned. No split, hole, double flap, extra tape, exposed bezel, strong wind, installation, speech, text or logo.</x:v>
+        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str">
-        <x:v>Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="M6" s="16" t="str">
-        <x:v>camera orbit, broken film, tape overhang, presenter blocking television, extra plastic layer</x:v>
+        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
       </x:c>
       <x:c r="N6" s="16" t="str">
-        <x:v>b3b654812d2d</x:v>
+        <x:v>fc5af9625de9</x:v>
       </x:c>
       <x:c r="O6" s="16" t="str">
         <x:v>通过</x:v>
@@ -866,7 +866,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="W6" s="16" t="str">
-        <x:v>completed</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="X6" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
@@ -875,10 +875,10 @@
         <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Z6" s="16" t="str">
-        <x:v>220888f5910eebd3</x:v>
+        <x:v>f00122b818f63193</x:v>
       </x:c>
       <x:c r="AA6" s="16" t="str">
-        <x:v>159e41806fbf71f6</x:v>
+        <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -892,7 +892,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f8ee893e244c3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c76b0b66ab42f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1151,25 +1151,25 @@
         <x:v>v01-s01</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 65-inch ultra-thin wall-mounted flat panel. Environment: bright Scandinavian living room under repainting. Coverage state: fully covered by a taut rectangular clear film curtain. Shot scale: wide full-wall shot. Camera motion: slow left-to-right lateral slider. Person or work state: no person; completed protection state. Opening visual and product geometry: Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：65英寸超薄壁挂平板电视。 环境场景：正在重新粉刷的明亮北欧风客厅。覆盖状态：一整张绷紧的矩形透明膜完整覆盖电视，并在四周留出清晰边界。 镜头景别：正面墙体全景；镜头运动：镜头从左向右缓慢横移。 人物或施工状态：无人物，防护施工已经完成。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。 动态过程：以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>Maintain the approved Scandinavian living-room keyframe and exact integrated product geometry. The 65-inch television stays fully behind one continuous clear film sheet; the yellow wall tape stays bonded across the complete film top edge with aligned endpoints. Execute a slow left-to-right lateral slider move that reveals mild parallax between the oak console and pale wall. Only tiny natural surface shimmer may occur in the film; no tear, opening, doubled flap, loose tape, uncovered television, person, installation action, transformation, flicker, text or logo.</x:v>
+        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>Use the reference only as the exact geometry standard for one integrated yellow tape and one intact transparent film sheet; create a clearly different setting and television. Photorealistic vertical commercial photograph of a 65-inch ultra-thin wall-mounted flat-panel television on a smooth pale-gray plaster wall in a bright Scandinavian living room being repainted. Include an oak console, covered sofa edge and folded canvas drop cloth in the wider background. One finite straight yellow masking-tape strip is adhered to the wall 12 centimeters above the television. Its square endpoints align exactly with the left and right vertical edges of one single transparent PE sheet permanently bonded along the tape's full lower edge. No tape extends beyond the film. The unbroken clear sheet hangs as one taut rectangular curtain in front of and completely beyond all four edges of the television, proven by soft reflections across the whole black screen and bezel. No hole, slit, split, flap, doubled layer, missing corner or detached tape. No person or hands. Wide full-wall composition, front-facing eye level, bright cool daylight, clean realistic renovation advertising, no text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
-        <x:v>broken film, split plastic, extra tape, exposed screen, tape on television, duplicate sheet</x:v>
+        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="G4" s="16" t="str">
-        <x:v>a432a56c0d26223d</x:v>
+        <x:v>4608463e01bf6f70</x:v>
       </x:c>
       <x:c r="H4" s="16" t="str">
-        <x:v>989be0d00589988c</x:v>
+        <x:v>365df2c1d064cfcd</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="300" customHeight="1">
@@ -1177,25 +1177,25 @@
         <x:v>v02-s01</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 43-inch compact wall-mounted flat panel. Environment: warm boutique-hotel bedroom renovation. Coverage state: fully covered with softly draped side and lower margins. Shot scale: three-quarter medium shot from the right. Camera motion: slow rightward dolly with restrained parallax. Person or work state: professional painter kneeling at frame left and visually inspecting without touching. Opening visual and product geometry: Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：43英寸紧凑型壁挂平板电视。 环境场景：正在翻新的暖色精品酒店客房。覆盖状态：透明膜完整覆盖电视，侧边和下沿呈轻微自然垂坠。 镜头景别：从右侧拍摄的四分之三中景；镜头运动：镜头缓慢向右移动，产生克制的空间视差。 人物或施工状态：专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。 动态过程：以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>Preserve the boutique-hotel bedroom, compact television, kneeling painter and the approved one-piece tape-film structure. Move the camera slowly to the right for restrained parallax across the walnut desk. The painter only shifts his gaze from the lower film margin to the yellow tape and gives one small satisfied nod; he never touches the product. The transparent sheet remains one intact layer covering the complete television, and both film edges remain aligned with the tape endpoints. No tear, flap, second layer, tape movement, installation, exposed screen, body occlusion, lip movement, text or logo.</x:v>
+        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>Use the reference only for the non-negotiable same-width tape-and-film connection; change the television size, room, camera angle and human state. Photorealistic vertical commercial photograph in a warm boutique-hotel bedroom under renovation. A compact 43-inch black television is wall mounted above a narrow walnut desk on a smooth cream wall. One finite yellow masking-tape strip is fixed to the wall 10 centimeters above it. One intact transparent PE film sheet begins exactly at both tape endpoints and is permanently connected across the tape's full lower edge. The film is one continuous layer in front of the television, with soft side and lower margins covering 100 percent of screen and bezel. A professional European male painter in clean white workwear kneels at far frame left, looking toward the protected lower edge without touching the film or tape; his body never blocks the product. Three-quarter medium view from the right, warm practical bedside lighting plus soft daylight. No hole, opening, split, flap, second sheet, extra tape, exposed television, text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>hands touching film, torn plastic, extra tape, person blocking product, exposed television</x:v>
+        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="G5" s="16" t="str">
-        <x:v>c6ef5a34bdd7a12b</x:v>
+        <x:v>4cb8aea4db242032</x:v>
       </x:c>
       <x:c r="H5" s="16" t="str">
-        <x:v>3d95e6b36115d38a</x:v>
+        <x:v>8c9b3e0b2372ea58</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="300" customHeight="1">
@@ -1203,25 +1203,25 @@
         <x:v>v03-s01</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Create a 10-second vertical 9:16 photorealistic renovation product demonstration video. Object: television; form: 75-inch wide wall-mounted flat panel. Environment: industrial loft media room with smooth white mounting panel. Coverage state: fully covered with broad transparent margins and lightly tensioned lower edge. Shot scale: low-angle wide shot. Camera motion: gentle upward tilt from console to tape line. Person or work state: standing painter at far right pointing beside the protected area. Opening visual and product geometry: Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark. Throughout the entire shot, the transparent PE film must remain one continuous intact sheet permanently bonded along the full lower edge of one straight yellow masking-tape strip. Keep the target object fully behind the film with no holes, tears, splits, duplicated film, extra tape, exposed object, text, logo or watermark.</x:v>
+        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：75英寸超宽壁挂平板电视。 环境场景：带白色安装墙面的工业风阁楼影音区。覆盖状态：宽幅透明膜完整覆盖电视，左右留出宽边，下沿轻微绷紧。 镜头景别：低机位广角镜头；镜头运动：镜头从下方电视柜缓慢向上抬升至黄色胶带。 人物或施工状态：专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。 动态过程：以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>Keep the industrial loft, 75-inch television, standing painter and full-width one-piece film installation unchanged. Begin low on the black metal console and perform a gentle upward camera tilt ending on the straight yellow tape line. The painter makes one restrained open-palm presentation gesture beside the film boundary without touching it. Throughout the tilt the television remains fully behind one continuous transparent sheet with broad margins; tape and film endpoints stay aligned. No split, hole, double flap, extra tape, exposed bezel, strong wind, installation, speech, text or logo.</x:v>
+        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
-        <x:v>Use the reference solely as the exact integrated product geometry; make the object, environment, framing and worker state visibly different. Photorealistic vertical commercial photograph of a very wide 75-inch wall-mounted flat-panel television centered on a large smooth white mounting panel set into an industrial loft media room with dark brick visible at both sides and a black metal console below. A single finite yellow masking-tape strip is adhered horizontally to the white panel 15 centimeters above the television. Exactly one broad intact transparent PE film sheet is bonded continuously to the tape's entire lower edge; film and tape have identical left and right endpoints. The clear sheet passes in front of the entire wide television and extends beyond both side edges and below the bottom bezel as one readable layer. A professional European painter stands at the far right outside the film boundary and points beside, not at or through, the protected area. Low-angle wide composition emphasizing the broad rectangular coverage. No broken plastic, seam, opening, duplicated sheet, tape overhang, person occlusion, text, logo or watermark.</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>camera orbit, broken film, tape overhang, presenter blocking television, extra plastic layer</x:v>
+        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
         <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>220888f5910eebd3</x:v>
+        <x:v>f00122b818f63193</x:v>
       </x:c>
       <x:c r="H6" s="16" t="str">
-        <x:v>159e41806fbf71f6</x:v>
+        <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1230,7 +1230,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3ef628e33604f7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83edd716d26341c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1335,7 +1335,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f34302527ad4904"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378f018ac7f046ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: remove fabricated text-to-video fields
</commit_message>
<xml_diff>
--- a/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
+++ b/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Ra02494dbf7224a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R792018fec5f84ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R639119724e834264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="Rdb62b6ab7e824234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Rb427dd3323984669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R21f612808be442eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R368e25764fc94764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R5a08da2bc5b24ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,8 +180,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVVideoStrategy" displayName="TVVideoStrategy" ref="A3:AA6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="27">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVVideoStrategy" displayName="TVVideoStrategy" ref="A3:Y6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="25">
     <x:tableColumn id="1" name="案例ID"/>
     <x:tableColumn id="2" name="案例名称"/>
     <x:tableColumn id="3" name="物体种类"/>
@@ -191,40 +191,36 @@
     <x:tableColumn id="7" name="镜头景别"/>
     <x:tableColumn id="8" name="镜头运动"/>
     <x:tableColumn id="9" name="人物/施工状态"/>
-    <x:tableColumn id="10" name="完整文生视频提示词"/>
-    <x:tableColumn id="11" name="图生视频提示词"/>
-    <x:tableColumn id="12" name="首帧提示词"/>
-    <x:tableColumn id="13" name="负面提示词"/>
-    <x:tableColumn id="14" name="唯一组合指纹"/>
-    <x:tableColumn id="15" name="首帧状态"/>
-    <x:tableColumn id="16" name="视频状态"/>
-    <x:tableColumn id="17" name="图片哈希"/>
-    <x:tableColumn id="18" name="视频哈希"/>
-    <x:tableColumn id="19" name="图片模型"/>
-    <x:tableColumn id="20" name="视频模型"/>
-    <x:tableColumn id="21" name="预计视频费用（元）"/>
-    <x:tableColumn id="22" name="生成秒数"/>
-    <x:tableColumn id="23" name="任务状态"/>
-    <x:tableColumn id="24" name="参考图片"/>
-    <x:tableColumn id="25" name="项目相对路径"/>
-    <x:tableColumn id="26" name="文生视频提示词哈希"/>
-    <x:tableColumn id="27" name="图生视频提示词哈希"/>
+    <x:tableColumn id="10" name="视频生成提示词（图生视频）"/>
+    <x:tableColumn id="11" name="首帧提示词（文生图）"/>
+    <x:tableColumn id="12" name="负面提示词"/>
+    <x:tableColumn id="13" name="唯一组合指纹"/>
+    <x:tableColumn id="14" name="首帧状态"/>
+    <x:tableColumn id="15" name="视频状态"/>
+    <x:tableColumn id="16" name="图片哈希"/>
+    <x:tableColumn id="17" name="视频哈希"/>
+    <x:tableColumn id="18" name="图片模型"/>
+    <x:tableColumn id="19" name="视频模型"/>
+    <x:tableColumn id="20" name="预计视频费用（元）"/>
+    <x:tableColumn id="21" name="生成秒数"/>
+    <x:tableColumn id="22" name="任务状态"/>
+    <x:tableColumn id="23" name="参考图片"/>
+    <x:tableColumn id="24" name="项目相对路径"/>
+    <x:tableColumn id="25" name="视频提示词哈希"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:H6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:F6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="案例ID"/>
-    <x:tableColumn id="2" name="完整文生视频提示词"/>
-    <x:tableColumn id="3" name="图生视频提示词"/>
-    <x:tableColumn id="4" name="首帧提示词"/>
-    <x:tableColumn id="5" name="负面提示词"/>
-    <x:tableColumn id="6" name="参考图片"/>
-    <x:tableColumn id="7" name="文生视频提示词哈希"/>
-    <x:tableColumn id="8" name="图生视频提示词哈希"/>
+    <x:tableColumn id="2" name="视频生成提示词（图生视频）"/>
+    <x:tableColumn id="3" name="首帧提示词（文生图）"/>
+    <x:tableColumn id="4" name="负面提示词"/>
+    <x:tableColumn id="5" name="参考图片"/>
+    <x:tableColumn id="6" name="视频提示词哈希"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -449,104 +445,96 @@
     <x:col min="10" max="10" width="70" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="70" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="70" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="70" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="16" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="38" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="16" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="16" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="34" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="38" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="N1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="U1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="V1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="W1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="X1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
       <x:c r="Y1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
-      </x:c>
-      <x:c r="Z1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
-      </x:c>
-      <x:c r="AA1" s="3" t="str">
-        <x:v>电视视频策略库｜七个维度 + 一条组合对应一条文生视频提示词</x:v>
+        <x:v>电视视频策略库｜七个维度 + 首帧提示词 + 实际视频生成提示词</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -578,58 +566,52 @@
         <x:v>人物/施工状态</x:v>
       </x:c>
       <x:c r="J3" s="15" t="str">
-        <x:v>完整文生视频提示词</x:v>
+        <x:v>视频生成提示词（图生视频）</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>图生视频提示词</x:v>
+        <x:v>首帧提示词（文生图）</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
-        <x:v>首帧提示词</x:v>
+        <x:v>负面提示词</x:v>
       </x:c>
       <x:c r="M3" s="15" t="str">
-        <x:v>负面提示词</x:v>
+        <x:v>唯一组合指纹</x:v>
       </x:c>
       <x:c r="N3" s="15" t="str">
-        <x:v>唯一组合指纹</x:v>
+        <x:v>首帧状态</x:v>
       </x:c>
       <x:c r="O3" s="15" t="str">
-        <x:v>首帧状态</x:v>
+        <x:v>视频状态</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>视频状态</x:v>
+        <x:v>图片哈希</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
-        <x:v>图片哈希</x:v>
+        <x:v>视频哈希</x:v>
       </x:c>
       <x:c r="R3" s="15" t="str">
-        <x:v>视频哈希</x:v>
+        <x:v>图片模型</x:v>
       </x:c>
       <x:c r="S3" s="15" t="str">
-        <x:v>图片模型</x:v>
+        <x:v>视频模型</x:v>
       </x:c>
       <x:c r="T3" s="15" t="str">
-        <x:v>视频模型</x:v>
+        <x:v>预计视频费用（元）</x:v>
       </x:c>
       <x:c r="U3" s="15" t="str">
-        <x:v>预计视频费用（元）</x:v>
+        <x:v>生成秒数</x:v>
       </x:c>
       <x:c r="V3" s="15" t="str">
-        <x:v>生成秒数</x:v>
+        <x:v>任务状态</x:v>
       </x:c>
       <x:c r="W3" s="15" t="str">
-        <x:v>任务状态</x:v>
+        <x:v>参考图片</x:v>
       </x:c>
       <x:c r="X3" s="15" t="str">
-        <x:v>参考图片</x:v>
-      </x:c>
-      <x:c r="Y3" s="15" t="str">
         <x:v>项目相对路径</x:v>
       </x:c>
-      <x:c r="Z3" s="15" t="str">
-        <x:v>文生视频提示词哈希</x:v>
-      </x:c>
-      <x:c r="AA3" s="11" t="str">
-        <x:v>图生视频提示词哈希</x:v>
+      <x:c r="Y3" s="11" t="str">
+        <x:v>视频提示词哈希</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="300" customHeight="1">
@@ -661,57 +643,51 @@
         <x:v>无人物，防护施工已经完成</x:v>
       </x:c>
       <x:c r="J4" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：65英寸超薄壁挂平板电视。 环境场景：正在重新粉刷的明亮北欧风客厅。覆盖状态：一整张绷紧的矩形透明膜完整覆盖电视，并在四周留出清晰边界。 镜头景别：正面墙体全景；镜头运动：镜头从左向右缓慢横移。 人物或施工状态：无人物，防护施工已经完成。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。 动态过程：以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
       </x:c>
       <x:c r="K4" s="16" t="str">
-        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
       </x:c>
       <x:c r="L4" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
+        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
       </x:c>
       <x:c r="M4" s="16" t="str">
-        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
+        <x:v>a2db2b40b93d</x:v>
       </x:c>
       <x:c r="N4" s="16" t="str">
-        <x:v>a2db2b40b93d</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O4" s="16" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="P4" s="16" t="str">
-        <x:v>通过</x:v>
+        <x:v>5a1fe65799bc295023a3214271fca0dc2e937204ba29e1fb377d2f1808602caf</x:v>
       </x:c>
       <x:c r="Q4" s="16" t="str">
-        <x:v>5a1fe65799bc295023a3214271fca0dc2e937204ba29e1fb377d2f1808602caf</x:v>
+        <x:v>e1cbb570af138da14ef24c8185c9ded84e2c9005570140ac3b2f8a9d6961889b</x:v>
       </x:c>
       <x:c r="R4" s="16" t="str">
-        <x:v>e1cbb570af138da14ef24c8185c9ded84e2c9005570140ac3b2f8a9d6961889b</x:v>
+        <x:v>seedream-5.0-lite</x:v>
       </x:c>
       <x:c r="S4" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="T4" s="16" t="str">
         <x:v>grok-imagine-video-1.5-fast</x:v>
       </x:c>
-      <x:c r="U4" s="20" t="n">
+      <x:c r="T4" s="20" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="V4" s="16" t="n">
+      <x:c r="U4" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="V4" s="16" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
       <x:c r="W4" s="16" t="str">
-        <x:v>已完成</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="X4" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y4" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-      <x:c r="Z4" s="16" t="str">
-        <x:v>4608463e01bf6f70</x:v>
-      </x:c>
-      <x:c r="AA4" s="16" t="str">
         <x:v>365df2c1d064cfcd</x:v>
       </x:c>
     </x:row>
@@ -744,57 +720,51 @@
         <x:v>专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品</x:v>
       </x:c>
       <x:c r="J5" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：43英寸紧凑型壁挂平板电视。 环境场景：正在翻新的暖色精品酒店客房。覆盖状态：透明膜完整覆盖电视，侧边和下沿呈轻微自然垂坠。 镜头景别：从右侧拍摄的四分之三中景；镜头运动：镜头缓慢向右移动，产生克制的空间视差。 人物或施工状态：专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。 动态过程：以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
       </x:c>
       <x:c r="K5" s="16" t="str">
-        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
+        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
       </x:c>
       <x:c r="M5" s="16" t="str">
-        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
+        <x:v>9d72917b4125</x:v>
       </x:c>
       <x:c r="N5" s="16" t="str">
-        <x:v>9d72917b4125</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O5" s="16" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="P5" s="16" t="str">
-        <x:v>通过</x:v>
+        <x:v>0303b24d530d619f3aed59ac14065486768a84e9a52c98a21a4b053bd4db78bc</x:v>
       </x:c>
       <x:c r="Q5" s="16" t="str">
-        <x:v>0303b24d530d619f3aed59ac14065486768a84e9a52c98a21a4b053bd4db78bc</x:v>
+        <x:v>c3db73e0a1871d0c6ec6e6918d7d6b3fef82e941b093320cfe58808bea9c58b7</x:v>
       </x:c>
       <x:c r="R5" s="16" t="str">
-        <x:v>c3db73e0a1871d0c6ec6e6918d7d6b3fef82e941b093320cfe58808bea9c58b7</x:v>
+        <x:v>seedream-5.0-lite</x:v>
       </x:c>
       <x:c r="S5" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="T5" s="16" t="str">
         <x:v>grok-imagine-video-1.5-fast</x:v>
       </x:c>
-      <x:c r="U5" s="20" t="n">
+      <x:c r="T5" s="20" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="V5" s="16" t="n">
+      <x:c r="U5" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="V5" s="16" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
       <x:c r="W5" s="16" t="str">
-        <x:v>已完成</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="X5" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y5" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-      <x:c r="Z5" s="16" t="str">
-        <x:v>4cb8aea4db242032</x:v>
-      </x:c>
-      <x:c r="AA5" s="16" t="str">
         <x:v>8c9b3e0b2372ea58</x:v>
       </x:c>
     </x:row>
@@ -827,72 +797,66 @@
         <x:v>专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势</x:v>
       </x:c>
       <x:c r="J6" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：75英寸超宽壁挂平板电视。 环境场景：带白色安装墙面的工业风阁楼影音区。覆盖状态：宽幅透明膜完整覆盖电视，左右留出宽边，下沿轻微绷紧。 镜头景别：低机位广角镜头；镜头运动：镜头从下方电视柜缓慢向上抬升至黄色胶带。 人物或施工状态：专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。 动态过程：以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
       </x:c>
       <x:c r="K6" s="16" t="str">
-        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
+        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
       </x:c>
       <x:c r="M6" s="16" t="str">
-        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
+        <x:v>fc5af9625de9</x:v>
       </x:c>
       <x:c r="N6" s="16" t="str">
-        <x:v>fc5af9625de9</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O6" s="16" t="str">
-        <x:v>通过</x:v>
+        <x:v>淘汰</x:v>
       </x:c>
       <x:c r="P6" s="16" t="str">
-        <x:v>淘汰</x:v>
+        <x:v>9fbc6f466b567258e7d6339a36bc6db7522e8b1c60a3d3e55c006dd0606b9060</x:v>
       </x:c>
       <x:c r="Q6" s="16" t="str">
-        <x:v>9fbc6f466b567258e7d6339a36bc6db7522e8b1c60a3d3e55c006dd0606b9060</x:v>
+        <x:v>93ae4e3521b49c08de0e3073cdcfb5313fe8e52aabcf823bb6722e7fcd8bb870</x:v>
       </x:c>
       <x:c r="R6" s="16" t="str">
-        <x:v>93ae4e3521b49c08de0e3073cdcfb5313fe8e52aabcf823bb6722e7fcd8bb870</x:v>
+        <x:v>seedream-5.0-lite</x:v>
       </x:c>
       <x:c r="S6" s="16" t="str">
-        <x:v>seedream-5.0-lite</x:v>
-      </x:c>
-      <x:c r="T6" s="16" t="str">
         <x:v>grok-imagine-video-1.5-fast</x:v>
       </x:c>
-      <x:c r="U6" s="20" t="n">
+      <x:c r="T6" s="20" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="V6" s="16" t="n">
+      <x:c r="U6" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="V6" s="16" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
       <x:c r="W6" s="16" t="str">
-        <x:v>已完成</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="X6" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y6" s="16" t="str">
-        <x:v>03_视频项目/防尘膜短视频/08_场景单元/06_电视_差异化场景/技术记录（不用看）</x:v>
-      </x:c>
-      <x:c r="Z6" s="16" t="str">
-        <x:v>f00122b818f63193</x:v>
-      </x:c>
-      <x:c r="AA6" s="16" t="str">
         <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AA1"/>
+    <x:mergeCell ref="A1:Y1"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="O4:P6">
+  <x:conditionalFormatting sqref="N4:O6">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="淘汰"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="待"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c76b0b66ab42f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91fa11bb28c94539"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -967,7 +931,7 @@
         <x:v>唯一七维组合数</x:v>
       </x:c>
       <x:c r="B5" s="17" t="n">
-        <x:f>COUNTA('视频策略库'!$N$4:$N$100)</x:f>
+        <x:f>COUNTA('视频策略库'!$M$4:$M$100)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
@@ -980,7 +944,7 @@
         <x:v>首帧通过数</x:v>
       </x:c>
       <x:c r="B6" s="17" t="n">
-        <x:f>COUNTIF('视频策略库'!$O$4:$O$100,"通过")</x:f>
+        <x:f>COUNTIF('视频策略库'!$N$4:$N$100,"通过")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
@@ -993,7 +957,7 @@
         <x:v>视频通过数</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
-        <x:f>COUNTIF('视频策略库'!$P$4:$P$100,"通过")</x:f>
+        <x:f>COUNTIF('视频策略库'!$O$4:$O$100,"通过")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
@@ -1006,7 +970,7 @@
         <x:v>预计视频费用（元）</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:f>ROUND(SUM('视频策略库'!$U$4:$U$100),2)</x:f>
+        <x:f>ROUND(SUM('视频策略库'!$T$4:$T$100),2)</x:f>
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
@@ -1049,7 +1013,7 @@
         <x:v>台账定位</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>主表逐行列出七维组合及其完整文生视频提示词；统计页仅用于辅助查看</x:v>
+        <x:v>主表逐行列出七维组合、首帧提示词和实际使用的视频生成提示词；统计页仅用于辅助查看</x:v>
       </x:c>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="19"/>
@@ -1087,37 +1051,29 @@
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="70" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>电视提示词档案｜区分文生视频、图生视频与首帧提示词</x:v>
+        <x:v>电视提示词档案｜真实流水线：首帧文生图 → 图生视频</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -1125,25 +1081,19 @@
         <x:v>案例ID</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>完整文生视频提示词</x:v>
+        <x:v>视频生成提示词（图生视频）</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>图生视频提示词</x:v>
+        <x:v>首帧提示词（文生图）</x:v>
       </x:c>
       <x:c r="D3" s="15" t="str">
-        <x:v>首帧提示词</x:v>
+        <x:v>负面提示词</x:v>
       </x:c>
       <x:c r="E3" s="15" t="str">
-        <x:v>负面提示词</x:v>
-      </x:c>
-      <x:c r="F3" s="15" t="str">
         <x:v>参考图片</x:v>
       </x:c>
-      <x:c r="G3" s="15" t="str">
-        <x:v>文生视频提示词哈希</x:v>
-      </x:c>
-      <x:c r="H3" s="11" t="str">
-        <x:v>图生视频提示词哈希</x:v>
+      <x:c r="F3" s="11" t="str">
+        <x:v>视频提示词哈希</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="300" customHeight="1">
@@ -1151,24 +1101,18 @@
         <x:v>v01-s01</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：65英寸超薄壁挂平板电视。 环境场景：正在重新粉刷的明亮北欧风客厅。覆盖状态：一整张绷紧的矩形透明膜完整覆盖电视，并在四周留出清晰边界。 镜头景别：正面墙体全景；镜头运动：镜头从左向右缓慢横移。 人物或施工状态：无人物，防护施工已经完成。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。 动态过程：以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>以已批准的北欧客厅首帧为起点，保持65英寸壁挂电视、黄色胶带和一体式透明膜的结构完全不变。镜头从左向右缓慢横移，背景产生轻微视差；薄膜只能出现细微自然反光，不得移动、撕裂或消失。全程电视位于同一张透明膜后方，胶带与膜上沿连续连接，禁止人物进入、禁止安装动作、禁止新增胶带、禁止屏幕裸露、禁止文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在重新粉刷的明亮北欧风客厅内，一台65英寸超薄壁挂电视固定在浅色墙面。电视上方约12厘米的墙面粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张与胶带同宽的透明PE薄膜永久连接在胶带下沿，从胶带左右端点垂直向下展开，完整覆盖电视屏幕、边框及四周区域。薄膜必须位于电视前方，四边连续、无破口、无分叉、无第二层膜。画面无人物，正面墙体全景，冷色自然日光，真实装修广告质感，不出现文字、标识或水印。</x:v>
+        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
-        <x:v>破膜、裂口、分叉、双层膜、额外胶带、胶带贴在电视上、电视裸露、人物、安装动作、文字、标识、水印</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
-      </x:c>
-      <x:c r="G4" s="16" t="str">
-        <x:v>4608463e01bf6f70</x:v>
-      </x:c>
-      <x:c r="H4" s="16" t="str">
         <x:v>365df2c1d064cfcd</x:v>
       </x:c>
     </x:row>
@@ -1177,24 +1121,18 @@
         <x:v>v02-s01</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：43英寸紧凑型壁挂平板电视。 环境场景：正在翻新的暖色精品酒店客房。覆盖状态：透明膜完整覆盖电视，侧边和下沿呈轻微自然垂坠。 镜头景别：从右侧拍摄的四分之三中景；镜头运动：镜头缓慢向右移动，产生克制的空间视差。 人物或施工状态：专业欧美油漆工跪在画面左侧，只观察胶带边缘且不触碰产品。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。 动态过程：以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>以已批准的酒店客房首帧为起点，保持43英寸电视、跪姿油漆工以及胶带与薄膜的一体式结构不变。镜头缓慢向右移动，产生克制的空间视差；油漆工只把视线从薄膜下沿移向黄色胶带，并轻微点头，不触碰产品。薄膜始终是一整张连续材料，左右端点与胶带对齐，电视全程位于膜后。禁止撕裂、第二层膜、额外胶带、手部接触、屏幕裸露、人物遮挡、说话口型、文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：暖色精品酒店客房正在翻新，一台43英寸紧凑型壁挂电视安装在床头墙面。电视上方约10厘米的墙面粘贴一条笔直、长度有限的黄色美纹胶带；同宽透明PE薄膜永久连接在胶带整个下沿，作为一整张连续薄膜覆盖电视屏幕和边框，左右及下沿有轻微自然垂坠但没有开口。画面左侧是一名穿白色工作服的专业欧美男油漆工，跪姿观察胶带边缘，不接触、不遮挡产品。右侧四分之三中景，暖色实用灯光与柔和日光结合，无文字、标识或水印。</x:v>
+        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>手触碰薄膜、撕裂塑料、额外胶带、人物遮挡电视、电视裸露、双层膜、说话口型、文字、标识、水印</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
-      </x:c>
-      <x:c r="G5" s="16" t="str">
-        <x:v>4cb8aea4db242032</x:v>
-      </x:c>
-      <x:c r="H5" s="16" t="str">
         <x:v>8c9b3e0b2372ea58</x:v>
       </x:c>
     </x:row>
@@ -1203,34 +1141,28 @@
         <x:v>v03-s01</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>生成一条10秒、9:16竖屏、写实装修广告风格的视频。 物体种类：电视；物体形态：75英寸超宽壁挂平板电视。 环境场景：带白色安装墙面的工业风阁楼影音区。覆盖状态：宽幅透明膜完整覆盖电视，左右留出宽边，下沿轻微绷紧。 镜头景别：低机位广角镜头；镜头运动：镜头从下方电视柜缓慢向上抬升至黄色胶带。 人物或施工状态：专业欧美油漆工站在画面最右侧，在防护区域旁做展示手势。 首帧与产品结构：生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。 动态过程：以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。 全程硬性要求：透明PE薄膜必须始终是一整张连续完整的薄膜，并永久连接在同一条笔直黄色美纹胶带的整个下沿；目标物必须始终完整位于薄膜后方。不得出现孔洞、撕裂、分叉、重复薄膜、额外胶带、目标物裸露、文字、标识或水印。</x:v>
+        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>以已批准的工业风阁楼首帧为起点，保持75英寸电视、站立油漆工和整幅一体式防尘膜完全不变。镜头从黑色电视柜开始，缓慢向上抬升至黄色胶带；油漆工只在薄膜边界外做一次幅度很小的开放手掌展示动作。电视全程位于一整张连续透明膜后，膜面不得逐渐消失，胶带和薄膜端点始终对齐。禁止环绕运镜、破膜、双层膜、胶带悬空、额外胶带、电视裸露、人物遮挡、说话、文字和标识。</x:v>
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
-        <x:v>生成一张9:16竖屏写实商业摄影首帧：工业风阁楼影音区内，一台75英寸超宽壁挂电视安装在平整白色墙板上。电视上方约15厘米处粘贴一条水平、笔直、长度有限的黄色美纹胶带；一整张宽幅透明PE膜与胶带下沿全长永久连接，左右端点严格对齐，薄膜覆盖整台电视并在左右留下清晰宽边，下沿轻微绷紧。专业欧美男油漆工站在画面最右侧，在薄膜边界之外做开放手掌展示动作，不接触、不遮挡电视。低机位广角构图，工业风黑色电视柜位于前景，无文字、标识或水印。</x:v>
+        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>环绕运镜、透明膜消失、破膜、胶带超出薄膜、人物遮挡电视、额外塑料层、电视裸露、文字、标识、水印</x:v>
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
-      </x:c>
-      <x:c r="G6" s="16" t="str">
-        <x:v>f00122b818f63193</x:v>
-      </x:c>
-      <x:c r="H6" s="16" t="str">
         <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83edd716d26341c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86976c043b064be5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1335,7 +1267,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378f018ac7f046ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffa8e26d1a664480"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add seven planned TV strategy cases
</commit_message>
<xml_diff>
--- a/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
+++ b/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Rb427dd3323984669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R21f612808be442eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R368e25764fc94764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R5a08da2bc5b24ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Rf9dee5c2a98e4603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R45316bfa2f54428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="Rb97e2fe3547c4a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="Ree4e47010f5740db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVVideoStrategy" displayName="TVVideoStrategy" ref="A3:Y6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TVVideoStrategy" displayName="TVVideoStrategy" ref="A3:Y13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="案例ID"/>
     <x:tableColumn id="2" name="案例名称"/>
@@ -213,7 +213,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:F6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TVPromptArchive" displayName="TVPromptArchive" ref="A3:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="案例ID"/>
     <x:tableColumn id="2" name="视频生成提示词（图生视频）"/>
@@ -845,18 +845,515 @@
         <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
+    <x:row r="7" ht="300" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>v04-s01</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>电视案例04</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>55英寸安装在带脚轮移动支架上的平板电视</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>正在翻新的现代企业会议室</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>透明膜从电视后方墙面胶带垂至地面，完整覆盖电视、支架立柱和底座</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>左前方四分之三全身景</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>镜头沿对角线缓慢向前推进</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="str">
+        <x:v>两名施工人员停留在远处背景，不接近防护电视</x:v>
+      </x:c>
+      <x:c r="J7" s="16" t="str">
+        <x:v>以已批准的会议室首帧为起点，保持移动支架电视和整张墙面垂落薄膜的结构完全不变。镜头沿左前方向电视缓慢推进，产生轻微桌椅视差；远处施工人员只做低幅度整理工具动作，不靠近防护区域。透明膜全程从同一条黄色胶带连续垂至地面，电视、立柱和底座始终位于膜后。禁止脚轮移动、人物靠近、膜撕裂、额外胶带、屏幕裸露、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：现代企业会议室正在翻新，一台55英寸平板电视安装在带脚轮的黑色移动支架上，靠近浅灰墙面。电视后方墙面上粘贴一条比电视和支架更宽、长度有限且笔直的黄色美纹胶带；同宽透明PE膜永久连接在胶带整个下沿，作为一整张连续薄膜垂至地面，完整覆盖电视屏幕、边框、支架立柱和脚轮底座。两名施工人员位于远处背景，不接近或遮挡产品。左前方四分之三全身景，冷白会议室灯光，无破口、双层膜、额外胶带、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L7" s="16" t="str">
+        <x:v>电视支架移动、人物靠近产品、膜未覆盖底座、破膜、双层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M7" s="16" t="str">
+        <x:v>f9a2c9af6ddd</x:v>
+      </x:c>
+      <x:c r="N7" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O7" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P7" s="16" t="str"/>
+      <x:c r="Q7" s="16" t="str"/>
+      <x:c r="R7" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S7" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T7" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U7" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V7" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W7" s="16" t="str"/>
+      <x:c r="X7" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y7" s="16" t="str">
+        <x:v>c19ef482ca441899</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="300" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>v05-s01</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>电视案例05</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>32英寸小型超薄壁挂电视</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str">
+        <x:v>正在改造的明亮公寓厨房用餐区</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>窄幅透明膜从墙面胶带完整覆盖小电视，并延伸至下方餐边台前沿</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>正面中近景</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>镜头从黄色胶带缓慢向下移动至餐边台</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="str">
+        <x:v>专业欧美女油漆工站在画面右后方检查墙面，不触碰薄膜</x:v>
+      </x:c>
+      <x:c r="J8" s="16" t="str">
+        <x:v>以已批准的公寓厨房首帧为起点，保持32英寸电视、餐边台和一体式胶带薄膜结构不变。镜头从黄色胶带开始缓慢向下移动至被覆盖的餐边台前沿；右后方油漆工只转动视线检查墙面，不靠近产品。薄膜必须始终连续覆盖电视和台面边缘，不得收缩、分叉或产生第二层。禁止手部接触、额外胶带、屏幕裸露、说话、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K8" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：明亮公寓厨房用餐区正在改造，一台32英寸小型超薄电视壁挂在白色墙面，下面是浅木色餐边台。电视上方约10厘米处粘贴一条长度有限、笔直的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续覆盖电视屏幕和边框，并向下延伸覆盖餐边台前沿。专业欧美女油漆工站在画面右后方检查远离产品的墙面，不接触薄膜。正面中近景，明亮日光，无开口、无第二片膜、无额外胶带、无裸露电视、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L8" s="16" t="str">
+        <x:v>大尺寸电视、油漆工触碰薄膜、餐边台裸露、薄膜收缩、第二层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M8" s="16" t="str">
+        <x:v>4bde66615eef</x:v>
+      </x:c>
+      <x:c r="N8" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O8" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P8" s="16" t="str"/>
+      <x:c r="Q8" s="16" t="str"/>
+      <x:c r="R8" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S8" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T8" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U8" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V8" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W8" s="16" t="str"/>
+      <x:c r="X8" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y8" s="16" t="str">
+        <x:v>81e3b8a90c385099</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="300" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>v06-s01</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>电视案例06</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>85英寸超大会议室壁挂显示电视</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>高层写字楼大型董事会议室翻新区</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>超宽透明膜从整条墙面胶带垂落，完整覆盖大屏及其下方接口区域</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>正面对称超广角全景</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>镜头沿中轴线非常缓慢地向前推进</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="str">
+        <x:v>无人物，桌椅已移开，防护状态完整展示</x:v>
+      </x:c>
+      <x:c r="J9" s="16" t="str">
+        <x:v>以已批准的董事会议室首帧为起点，保持85英寸大屏和超宽一体式透明膜完全不变。镜头沿房间中轴线非常缓慢地向前推进，会议桌边缘产生对称视差；画面无人进入。薄膜全程保持完整矩形边界，黄色胶带与膜上沿等宽连续，大屏及接口区域始终位于膜后。禁止屏幕点亮、薄膜消失、胶带变长、第二层膜、人物、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K9" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：高层写字楼的大型董事会议室正在翻新，一台85英寸超大显示电视居中壁挂在深灰色装饰墙上，桌椅已移到两侧。电视上方约18厘米处粘贴一条超宽但长度有限、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续覆盖整块大屏、所有边框和下方接口区域，左右边界垂直清晰。无人物，正面对称超广角全景，窗外城市日光柔和，无薄膜缺角、胶带超出、第二层膜、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L9" s="16" t="str">
+        <x:v>屏幕点亮、薄膜消失、胶带超出薄膜、双层膜、人物进入、大屏裸露、接口裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M9" s="16" t="str">
+        <x:v>30db797cc154</x:v>
+      </x:c>
+      <x:c r="N9" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O9" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P9" s="16" t="str"/>
+      <x:c r="Q9" s="16" t="str"/>
+      <x:c r="R9" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S9" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T9" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U9" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V9" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W9" s="16" t="str"/>
+      <x:c r="X9" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y9" s="16" t="str">
+        <x:v>302b99bbb4073844</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="300" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>v07-s01</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>电视案例07</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>50英寸带中央底座的台式平板电视</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str">
+        <x:v>正在粉刷的学校多媒体教室</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="str">
+        <x:v>透明膜从黑板旁墙面胶带垂下，完整覆盖电视、中央底座和讲台台面</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>右前方环境中景</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="str">
+        <x:v>镜头从右前方向左后方缓慢侧移</x:v>
+      </x:c>
+      <x:c r="I10" s="16" t="str">
+        <x:v>一名专业欧美油漆工站在远端手持滚筒，保持静止</x:v>
+      </x:c>
+      <x:c r="J10" s="16" t="str">
+        <x:v>以已批准的多媒体教室首帧为起点，保持台式电视、中央底座、讲台和整张透明膜结构不变。镜头从右前方向左后方缓慢侧移，课桌产生轻微视差；远端油漆工保持静止，只轻微调整握持滚筒的姿势。薄膜全程覆盖电视、底座和讲台台面，胶带和膜左右端点始终对齐。禁止人物走动、滚筒接触薄膜、底座裸露、第二层膜、额外胶带、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K10" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：学校多媒体教室正在粉刷，一台50英寸带中央底座的台式平板电视放在木质讲台上，靠近黑板旁的白墙。墙面上粘贴一条覆盖电视和讲台宽度的有限黄色美纹胶带；同宽透明PE膜永久连接在胶带下沿，作为一整张连续薄膜完整覆盖电视、中央底座和讲台台面。专业欧美油漆工站在远端手持滚筒并保持静止，不接近防护区。右前方环境中景，柔和教室日光，无薄膜开口、无额外胶带、无电视裸露、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L10" s="16" t="str">
+        <x:v>人物走动、滚筒触碰薄膜、中央底座裸露、讲台裸露、双层膜、额外胶带、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M10" s="16" t="str">
+        <x:v>d2e0e1c22b55</x:v>
+      </x:c>
+      <x:c r="N10" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O10" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P10" s="16" t="str"/>
+      <x:c r="Q10" s="16" t="str"/>
+      <x:c r="R10" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S10" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T10" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U10" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V10" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W10" s="16" t="str"/>
+      <x:c r="X10" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y10" s="16" t="str">
+        <x:v>9c15598cfb500bba</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="300" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>v08-s01</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>电视案例08</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>21英寸复古显像管电视</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>正在翻新的老式砖墙公寓客厅</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>透明膜从砖墙胶带垂下，完整包覆厚电视机身和下方矮柜</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>低机位近景</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>镜头以极慢速度向复古电视正面推进</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="str">
+        <x:v>无人物，防护施工完成，周围工具静置</x:v>
+      </x:c>
+      <x:c r="J11" s="16" t="str">
+        <x:v>以已批准的复古公寓首帧为起点，保持显像管电视、木质矮柜和一体式防护膜结构不变。镜头以极慢速度向电视正面推进，透明膜只出现柔和反光，凸屏和厚机身始终完整位于同一张膜后。画面无人进入，工具保持静止。禁止电视变成平板、屏幕点亮、薄膜穿入机身、第二层膜、额外胶带、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K11" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在翻新的老式砖墙公寓客厅内，一台21英寸复古显像管电视放在深色木质矮柜上，机身厚重、屏幕微凸。电视上方砖墙粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续包覆显像管电视的顶部、凸屏、厚侧面和矮柜前沿。无人物，装修工具静置在远处，低机位近景，暖色窗光，无膜面开口、无重复薄膜、无额外胶带、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L11" s="16" t="str">
+        <x:v>电视变成平板、屏幕点亮、薄膜穿模、厚机身裸露、双层膜、额外胶带、人物、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M11" s="16" t="str">
+        <x:v>27f48a0869e7</x:v>
+      </x:c>
+      <x:c r="N11" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O11" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P11" s="16" t="str"/>
+      <x:c r="Q11" s="16" t="str"/>
+      <x:c r="R11" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S11" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T11" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U11" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V11" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W11" s="16" t="str"/>
+      <x:c r="X11" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y11" s="16" t="str">
+        <x:v>8b75f65c54dcac7d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="300" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>v09-s01</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>电视案例09</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>48英寸户外防水壁挂电视</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str">
+        <x:v>正在重新涂装的有顶露台休闲区</x:v>
+      </x:c>
+      <x:c r="F12" s="16" t="str">
+        <x:v>抗风状态的透明膜绷紧覆盖电视，侧边固定清晰且下沿不飘起</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str">
+        <x:v>从左侧拍摄的环境中远景</x:v>
+      </x:c>
+      <x:c r="H12" s="16" t="str">
+        <x:v>镜头沿露台边缘从左向右平稳跟移</x:v>
+      </x:c>
+      <x:c r="I12" s="16" t="str">
+        <x:v>专业欧美油漆工站在画面右侧检查远处墙角，不触碰产品</x:v>
+      </x:c>
+      <x:c r="J12" s="16" t="str">
+        <x:v>以已批准的有顶露台首帧为起点，保持户外电视、油漆工和绷紧透明膜结构不变。镜头沿露台边缘从左向右平稳跟移，背景绿植产生轻微视差；膜面仅允许极小幅度自然颤动，下沿不得掀起，胶带与膜上沿必须持续连接。油漆工只检查远处墙角。禁止大风吹开薄膜、雨水、膜脱落、额外胶带、屏幕裸露、人物靠近、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K12" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：有顶露台休闲区正在重新涂装，一台48英寸户外防水电视壁挂在浅色外墙上，背景可见虚化绿植。电视上方约12厘米处粘贴一条有限长度、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，以轻微绷紧的抗风状态完整覆盖电视屏幕和边框，左右边界平直，下沿不飘起。专业欧美油漆工站在画面右侧检查远处墙角，不接触产品。左侧环境中远景，阴天柔光，无破膜、额外胶带、电视裸露、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L12" s="16" t="str">
+        <x:v>强风掀膜、膜脱落、雨水、胶带松脱、额外胶带、人物靠近、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M12" s="16" t="str">
+        <x:v>a9a49568cf79</x:v>
+      </x:c>
+      <x:c r="N12" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O12" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P12" s="16" t="str"/>
+      <x:c r="Q12" s="16" t="str"/>
+      <x:c r="R12" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S12" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T12" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U12" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V12" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W12" s="16" t="str"/>
+      <x:c r="X12" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y12" s="16" t="str">
+        <x:v>058501105e2b5b9a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="300" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>v10-s01</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>电视案例10</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>电视</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>55英寸嵌入式壁龛平板电视</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str">
+        <x:v>正在翻新的高端客厅整墙柜区域</x:v>
+      </x:c>
+      <x:c r="F13" s="16" t="str">
+        <x:v>透明膜从壁龛上沿柜板胶带垂下，完整封住电视壁龛开口</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>正面偏右的宽幅中景</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="str">
+        <x:v>镜头从壁龛细节缓慢向后拉远至整墙柜</x:v>
+      </x:c>
+      <x:c r="I13" s="16" t="str">
+        <x:v>专业欧美油漆工跪在画面右下方展示壁龛防护，不触碰薄膜</x:v>
+      </x:c>
+      <x:c r="J13" s="16" t="str">
+        <x:v>以已批准的整墙柜壁龛首帧为起点，保持嵌入式电视、壁龛、跪姿油漆工和完整透明膜结构不变。镜头从黄色胶带与壁龛上沿的连接细节开始，缓慢向后拉远，展示整墙柜范围；油漆工只做一次小幅开放手掌动作。透明膜全程完整封住壁龛开口，电视不得跑到膜前。禁止膜贴到电视屏幕、胶带悬空、壁龛开口裸露、第二层膜、额外胶带、说话、文字和标识。</x:v>
+      </x:c>
+      <x:c r="K13" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：高端客厅的整墙柜区域正在翻新，一台55英寸平板电视嵌入木质壁龛。壁龛开口上沿的水平柜板粘贴一条长度与开口相同、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，像透明帘幕一样完整封住整个壁龛开口，电视和壁龛内侧全部位于膜后。专业欧美油漆工跪在画面右下方，在薄膜边界外做展示手势，不触碰产品。正面偏右宽幅中景，暖色室内光，无膜面缺角、胶带悬空、额外胶带、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="L13" s="16" t="str">
+        <x:v>膜贴在电视屏幕上、胶带悬空、壁龛裸露、电视跑到膜前、双层膜、额外胶带、人物触碰、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="M13" s="16" t="str">
+        <x:v>51afb9a8bc5d</x:v>
+      </x:c>
+      <x:c r="N13" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="O13" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="P13" s="16" t="str"/>
+      <x:c r="Q13" s="16" t="str"/>
+      <x:c r="R13" s="16" t="str">
+        <x:v>seedream-5.0-lite</x:v>
+      </x:c>
+      <x:c r="S13" s="16" t="str">
+        <x:v>grok-imagine-video-1.5-fast</x:v>
+      </x:c>
+      <x:c r="T13" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U13" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V13" s="16" t="str">
+        <x:v>待生成</x:v>
+      </x:c>
+      <x:c r="W13" s="16" t="str"/>
+      <x:c r="X13" s="16" t="str">
+        <x:v>仅台账计划，尚未建立生成项目</x:v>
+      </x:c>
+      <x:c r="Y13" s="16" t="str">
+        <x:v>51e5b0d1d388fff7</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Y1"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="N4:O6">
+  <x:conditionalFormatting sqref="N4:O13">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="淘汰"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="待"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91fa11bb28c94539"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R482b238b295d4a5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -919,7 +1416,7 @@
       </x:c>
       <x:c r="B4" s="17" t="n">
         <x:f>COUNTA('视频策略库'!$A$4:$A$100)</x:f>
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C4" s="17"/>
       <x:c r="D4" s="17"/>
@@ -932,7 +1429,7 @@
       </x:c>
       <x:c r="B5" s="17" t="n">
         <x:f>COUNTA('视频策略库'!$M$4:$M$100)</x:f>
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
       <x:c r="D5" s="17"/>
@@ -967,11 +1464,11 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="17" t="str">
-        <x:v>预计视频费用（元）</x:v>
+        <x:v>全部案例预计视频费用（元）</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f>ROUND(SUM('视频策略库'!$T$4:$T$100),2)</x:f>
-        <x:v>1.8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
       <x:c r="D8" s="17"/>
@@ -998,10 +1495,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="19" t="str">
-        <x:v>机器执行源</x:v>
+        <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>技术记录（不用看）/project.json</x:v>
+        <x:v>已生成案例来自 project.json；待生成案例为台账中的策略计划</x:v>
       </x:c>
       <x:c r="C11" s="19"/>
       <x:c r="D11" s="19"/>
@@ -1013,7 +1510,7 @@
         <x:v>台账定位</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>主表逐行列出七维组合、首帧提示词和实际使用的视频生成提示词；统计页仅用于辅助查看</x:v>
+        <x:v>主表逐行列出七维组合、首帧提示词和对应的视频生成提示词；待生成案例不计为已完成</x:v>
       </x:c>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="19"/>
@@ -1156,13 +1653,139 @@
         <x:v>c8b6b4f452377c85</x:v>
       </x:c>
     </x:row>
+    <x:row r="7" ht="300" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>v04-s01</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>以已批准的会议室首帧为起点，保持移动支架电视和整张墙面垂落薄膜的结构完全不变。镜头沿左前方向电视缓慢推进，产生轻微桌椅视差；远处施工人员只做低幅度整理工具动作，不靠近防护区域。透明膜全程从同一条黄色胶带连续垂至地面，电视、立柱和底座始终位于膜后。禁止脚轮移动、人物靠近、膜撕裂、额外胶带、屏幕裸露、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：现代企业会议室正在翻新，一台55英寸平板电视安装在带脚轮的黑色移动支架上，靠近浅灰墙面。电视后方墙面上粘贴一条比电视和支架更宽、长度有限且笔直的黄色美纹胶带；同宽透明PE膜永久连接在胶带整个下沿，作为一整张连续薄膜垂至地面，完整覆盖电视屏幕、边框、支架立柱和脚轮底座。两名施工人员位于远处背景，不接近或遮挡产品。左前方四分之三全身景，冷白会议室灯光，无破口、双层膜、额外胶带、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>电视支架移动、人物靠近产品、膜未覆盖底座、破膜、双层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str"/>
+      <x:c r="F7" s="16" t="str">
+        <x:v>c19ef482ca441899</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="300" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>v05-s01</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>以已批准的公寓厨房首帧为起点，保持32英寸电视、餐边台和一体式胶带薄膜结构不变。镜头从黄色胶带开始缓慢向下移动至被覆盖的餐边台前沿；右后方油漆工只转动视线检查墙面，不靠近产品。薄膜必须始终连续覆盖电视和台面边缘，不得收缩、分叉或产生第二层。禁止手部接触、额外胶带、屏幕裸露、说话、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：明亮公寓厨房用餐区正在改造，一台32英寸小型超薄电视壁挂在白色墙面，下面是浅木色餐边台。电视上方约10厘米处粘贴一条长度有限、笔直的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续覆盖电视屏幕和边框，并向下延伸覆盖餐边台前沿。专业欧美女油漆工站在画面右后方检查远离产品的墙面，不接触薄膜。正面中近景，明亮日光，无开口、无第二片膜、无额外胶带、无裸露电视、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>大尺寸电视、油漆工触碰薄膜、餐边台裸露、薄膜收缩、第二层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str"/>
+      <x:c r="F8" s="16" t="str">
+        <x:v>81e3b8a90c385099</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="300" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>v06-s01</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>以已批准的董事会议室首帧为起点，保持85英寸大屏和超宽一体式透明膜完全不变。镜头沿房间中轴线非常缓慢地向前推进，会议桌边缘产生对称视差；画面无人进入。薄膜全程保持完整矩形边界，黄色胶带与膜上沿等宽连续，大屏及接口区域始终位于膜后。禁止屏幕点亮、薄膜消失、胶带变长、第二层膜、人物、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：高层写字楼的大型董事会议室正在翻新，一台85英寸超大显示电视居中壁挂在深灰色装饰墙上，桌椅已移到两侧。电视上方约18厘米处粘贴一条超宽但长度有限、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续覆盖整块大屏、所有边框和下方接口区域，左右边界垂直清晰。无人物，正面对称超广角全景，窗外城市日光柔和，无薄膜缺角、胶带超出、第二层膜、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>屏幕点亮、薄膜消失、胶带超出薄膜、双层膜、人物进入、大屏裸露、接口裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str"/>
+      <x:c r="F9" s="16" t="str">
+        <x:v>302b99bbb4073844</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="300" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>v07-s01</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>以已批准的多媒体教室首帧为起点，保持台式电视、中央底座、讲台和整张透明膜结构不变。镜头从右前方向左后方缓慢侧移，课桌产生轻微视差；远端油漆工保持静止，只轻微调整握持滚筒的姿势。薄膜全程覆盖电视、底座和讲台台面，胶带和膜左右端点始终对齐。禁止人物走动、滚筒接触薄膜、底座裸露、第二层膜、额外胶带、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：学校多媒体教室正在粉刷，一台50英寸带中央底座的台式平板电视放在木质讲台上，靠近黑板旁的白墙。墙面上粘贴一条覆盖电视和讲台宽度的有限黄色美纹胶带；同宽透明PE膜永久连接在胶带下沿，作为一整张连续薄膜完整覆盖电视、中央底座和讲台台面。专业欧美油漆工站在远端手持滚筒并保持静止，不接近防护区。右前方环境中景，柔和教室日光，无薄膜开口、无额外胶带、无电视裸露、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>人物走动、滚筒触碰薄膜、中央底座裸露、讲台裸露、双层膜、额外胶带、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str"/>
+      <x:c r="F10" s="16" t="str">
+        <x:v>9c15598cfb500bba</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="300" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>v08-s01</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>以已批准的复古公寓首帧为起点，保持显像管电视、木质矮柜和一体式防护膜结构不变。镜头以极慢速度向电视正面推进，透明膜只出现柔和反光，凸屏和厚机身始终完整位于同一张膜后。画面无人进入，工具保持静止。禁止电视变成平板、屏幕点亮、薄膜穿入机身、第二层膜、额外胶带、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：正在翻新的老式砖墙公寓客厅内，一台21英寸复古显像管电视放在深色木质矮柜上，机身厚重、屏幕微凸。电视上方砖墙粘贴一条长度有限、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，连续包覆显像管电视的顶部、凸屏、厚侧面和矮柜前沿。无人物，装修工具静置在远处，低机位近景，暖色窗光，无膜面开口、无重复薄膜、无额外胶带、无文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>电视变成平板、屏幕点亮、薄膜穿模、厚机身裸露、双层膜、额外胶带、人物、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str"/>
+      <x:c r="F11" s="16" t="str">
+        <x:v>8b75f65c54dcac7d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="300" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>v09-s01</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>以已批准的有顶露台首帧为起点，保持户外电视、油漆工和绷紧透明膜结构不变。镜头沿露台边缘从左向右平稳跟移，背景绿植产生轻微视差；膜面仅允许极小幅度自然颤动，下沿不得掀起，胶带与膜上沿必须持续连接。油漆工只检查远处墙角。禁止大风吹开薄膜、雨水、膜脱落、额外胶带、屏幕裸露、人物靠近、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：有顶露台休闲区正在重新涂装，一台48英寸户外防水电视壁挂在浅色外墙上，背景可见虚化绿植。电视上方约12厘米处粘贴一条有限长度、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，以轻微绷紧的抗风状态完整覆盖电视屏幕和边框，左右边界平直，下沿不飘起。专业欧美油漆工站在画面右侧检查远处墙角，不接触产品。左侧环境中远景，阴天柔光，无破膜、额外胶带、电视裸露、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>强风掀膜、膜脱落、雨水、胶带松脱、额外胶带、人物靠近、屏幕裸露、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str"/>
+      <x:c r="F12" s="16" t="str">
+        <x:v>058501105e2b5b9a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="300" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>v10-s01</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>以已批准的整墙柜壁龛首帧为起点，保持嵌入式电视、壁龛、跪姿油漆工和完整透明膜结构不变。镜头从黄色胶带与壁龛上沿的连接细节开始，缓慢向后拉远，展示整墙柜范围；油漆工只做一次小幅开放手掌动作。透明膜全程完整封住壁龛开口，电视不得跑到膜前。禁止膜贴到电视屏幕、胶带悬空、壁龛开口裸露、第二层膜、额外胶带、说话、文字和标识。</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>生成一张9:16竖屏写实商业摄影首帧：高端客厅的整墙柜区域正在翻新，一台55英寸平板电视嵌入木质壁龛。壁龛开口上沿的水平柜板粘贴一条长度与开口相同、笔直完整的黄色美纹胶带；一整张同宽透明PE膜永久连接在胶带下沿，像透明帘幕一样完整封住整个壁龛开口，电视和壁龛内侧全部位于膜后。专业欧美油漆工跪在画面右下方，在薄膜边界外做展示手势，不触碰产品。正面偏右宽幅中景，暖色室内光，无膜面缺角、胶带悬空、额外胶带、文字、标识或水印。</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>膜贴在电视屏幕上、胶带悬空、壁龛裸露、电视跑到膜前、双层膜、额外胶带、人物触碰、文字、标识、水印</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str"/>
+      <x:c r="F13" s="16" t="str">
+        <x:v>51e5b0d1d388fff7</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86976c043b064be5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f6479f4c0c14f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1267,7 +1890,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffa8e26d1a664480"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70386a8d0c974529"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete seven-case TV production run
</commit_message>
<xml_diff>
--- a/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
+++ b/03_视频项目/防尘膜短视频/08_场景单元/素材策略台账/2026-07-17-差异化批次/电视素材策略台账.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="Rf9dee5c2a98e4603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R45316bfa2f54428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="Rb97e2fe3547c4a12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="Ree4e47010f5740db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频策略库" sheetId="1" r:id="R789b7859646345db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略总览" sheetId="2" r:id="R0dc211692bae4e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提示词档案" sheetId="3" r:id="R5cc2dd7ae91143f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="4" r:id="R655b7994a4c24e0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -227,7 +227,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TVRejects" displayName="TVRejects" ref="A3:D7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TVRejects" displayName="TVRejects" ref="A3:D8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="来源批次"/>
     <x:tableColumn id="2" name="案例/类型"/>
@@ -886,13 +886,17 @@
         <x:v>f9a2c9af6ddd</x:v>
       </x:c>
       <x:c r="N7" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O7" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P7" s="16" t="str"/>
-      <x:c r="Q7" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P7" s="16" t="str">
+        <x:v>cf9a5c536c55a2ce2ad65c69a12f5a9c83c5d7c15f60526e2fac70d6af40f70e</x:v>
+      </x:c>
+      <x:c r="Q7" s="16" t="str">
+        <x:v>6b7ff230f7f41919dd5eb652dc4ed3d8d2d7be9e308538fc35398c35b45ceb93</x:v>
+      </x:c>
       <x:c r="R7" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -906,11 +910,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V7" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W7" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W7" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X7" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y7" s="16" t="str">
         <x:v>c19ef482ca441899</x:v>
@@ -957,13 +963,17 @@
         <x:v>4bde66615eef</x:v>
       </x:c>
       <x:c r="N8" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O8" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P8" s="16" t="str"/>
-      <x:c r="Q8" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P8" s="16" t="str">
+        <x:v>7e4a469af25170ed35f030d275a870e7d1c8c828424485b549467823ab5c61df</x:v>
+      </x:c>
+      <x:c r="Q8" s="16" t="str">
+        <x:v>93e6c48bd1d0e29b8bcf2d5277adc7d45d9d43df63c9ed0fe23f72800d961810</x:v>
+      </x:c>
       <x:c r="R8" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -977,11 +987,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V8" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W8" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W8" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X8" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y8" s="16" t="str">
         <x:v>81e3b8a90c385099</x:v>
@@ -1028,13 +1040,17 @@
         <x:v>30db797cc154</x:v>
       </x:c>
       <x:c r="N9" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O9" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P9" s="16" t="str"/>
-      <x:c r="Q9" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P9" s="16" t="str">
+        <x:v>1db33c57983eb5178e3e7206149fa4a953fbffc2a2ec172ec616f804c1292310</x:v>
+      </x:c>
+      <x:c r="Q9" s="16" t="str">
+        <x:v>f07c48ff09460f6e55e2da4d9a5ae9d46611f60a29ba421672fcfdb42c14beff</x:v>
+      </x:c>
       <x:c r="R9" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -1048,11 +1064,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V9" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W9" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W9" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X9" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y9" s="16" t="str">
         <x:v>302b99bbb4073844</x:v>
@@ -1099,12 +1117,14 @@
         <x:v>d2e0e1c22b55</x:v>
       </x:c>
       <x:c r="N10" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>淘汰</x:v>
       </x:c>
       <x:c r="O10" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P10" s="16" t="str"/>
+        <x:v>未生成（首帧淘汰）</x:v>
+      </x:c>
+      <x:c r="P10" s="16" t="str">
+        <x:v>36cd2c006f6db56a3505dc261782b018a7c2cdf861e6cfb68ad619c266308343</x:v>
+      </x:c>
       <x:c r="Q10" s="16" t="str"/>
       <x:c r="R10" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
@@ -1113,17 +1133,19 @@
         <x:v>grok-imagine-video-1.5-fast</x:v>
       </x:c>
       <x:c r="T10" s="20" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="U10" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="V10" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W10" s="16" t="str"/>
+        <x:v>已拦截</x:v>
+      </x:c>
+      <x:c r="W10" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X10" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y10" s="16" t="str">
         <x:v>9c15598cfb500bba</x:v>
@@ -1170,13 +1192,17 @@
         <x:v>27f48a0869e7</x:v>
       </x:c>
       <x:c r="N11" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O11" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P11" s="16" t="str"/>
-      <x:c r="Q11" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P11" s="16" t="str">
+        <x:v>e92de995c24c905c9f77b81a776e6bf0a53185cc89ac9a6aded56eaa83b5988a</x:v>
+      </x:c>
+      <x:c r="Q11" s="16" t="str">
+        <x:v>f294b44c2ead48af899c925ee9afcccc0681a89668addf9951bf9a632d637b79</x:v>
+      </x:c>
       <x:c r="R11" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -1190,11 +1216,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V11" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W11" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W11" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X11" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y11" s="16" t="str">
         <x:v>8b75f65c54dcac7d</x:v>
@@ -1241,13 +1269,17 @@
         <x:v>a9a49568cf79</x:v>
       </x:c>
       <x:c r="N12" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O12" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P12" s="16" t="str"/>
-      <x:c r="Q12" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P12" s="16" t="str">
+        <x:v>45f7404282ffd5da651b854526c9d44bcb5357a0e0b80dfa242873a20fc31022</x:v>
+      </x:c>
+      <x:c r="Q12" s="16" t="str">
+        <x:v>d2fca356ad7145b647590cef3805204c9f7d424d8ce2ec72d27e1a34b7a650b7</x:v>
+      </x:c>
       <x:c r="R12" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -1261,11 +1293,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V12" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W12" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W12" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X12" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y12" s="16" t="str">
         <x:v>058501105e2b5b9a</x:v>
@@ -1312,13 +1346,17 @@
         <x:v>51afb9a8bc5d</x:v>
       </x:c>
       <x:c r="N13" s="16" t="str">
-        <x:v>待生成</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="O13" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="P13" s="16" t="str"/>
-      <x:c r="Q13" s="16" t="str"/>
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="P13" s="16" t="str">
+        <x:v>c0f259d2689e7e20e2812c8db84f5fbc217cf22a45d28a6de677aa66aed66fef</x:v>
+      </x:c>
+      <x:c r="Q13" s="16" t="str">
+        <x:v>b327f4624189aa769e70a2f7c2d8d8c4e1c8a9b4c9859c87abe0453be70ab164</x:v>
+      </x:c>
       <x:c r="R13" s="16" t="str">
         <x:v>seedream-5.0-lite</x:v>
       </x:c>
@@ -1332,11 +1370,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="V13" s="16" t="str">
-        <x:v>待生成</x:v>
-      </x:c>
-      <x:c r="W13" s="16" t="str"/>
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="W13" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="X13" s="16" t="str">
-        <x:v>仅台账计划，尚未建立生成项目</x:v>
+        <x:v>03_视频项目/防尘膜短视频/08_场景单元/08_电视_扩展七案例/技术记录（不用看）</x:v>
       </x:c>
       <x:c r="Y13" s="16" t="str">
         <x:v>51e5b0d1d388fff7</x:v>
@@ -1353,7 +1393,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R482b238b295d4a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81eb42d53f3544c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1442,7 +1482,7 @@
       </x:c>
       <x:c r="B6" s="17" t="n">
         <x:f>COUNTIF('视频策略库'!$N$4:$N$100,"通过")</x:f>
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
       <x:c r="D6" s="17"/>
@@ -1455,7 +1495,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('视频策略库'!$O$4:$O$100,"通过")</x:f>
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
       <x:c r="D7" s="17"/>
@@ -1468,7 +1508,7 @@
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f>ROUND(SUM('视频策略库'!$T$4:$T$100),2)</x:f>
-        <x:v>6</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
       <x:c r="D8" s="17"/>
@@ -1498,7 +1538,7 @@
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>已生成案例来自 project.json；待生成案例为台账中的策略计划</x:v>
+        <x:v>案例策略来自 project.json；生成状态来自首帧、视频哈希验收记录</x:v>
       </x:c>
       <x:c r="C11" s="19"/>
       <x:c r="D11" s="19"/>
@@ -1510,7 +1550,7 @@
         <x:v>台账定位</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>主表逐行列出七维组合、首帧提示词和对应的视频生成提示词；待生成案例不计为已完成</x:v>
+        <x:v>主表逐行列出七维组合、首帧提示词和对应的视频生成提示词；未通过质量门的案例不计为完成</x:v>
       </x:c>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="19"/>
@@ -1666,7 +1706,9 @@
       <x:c r="D7" s="16" t="str">
         <x:v>电视支架移动、人物靠近产品、膜未覆盖底座、破膜、双层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E7" s="16" t="str"/>
+      <x:c r="E7" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F7" s="16" t="str">
         <x:v>c19ef482ca441899</x:v>
       </x:c>
@@ -1684,7 +1726,9 @@
       <x:c r="D8" s="16" t="str">
         <x:v>大尺寸电视、油漆工触碰薄膜、餐边台裸露、薄膜收缩、第二层膜、额外胶带、屏幕裸露、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E8" s="16" t="str"/>
+      <x:c r="E8" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F8" s="16" t="str">
         <x:v>81e3b8a90c385099</x:v>
       </x:c>
@@ -1702,7 +1746,9 @@
       <x:c r="D9" s="16" t="str">
         <x:v>屏幕点亮、薄膜消失、胶带超出薄膜、双层膜、人物进入、大屏裸露、接口裸露、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E9" s="16" t="str"/>
+      <x:c r="E9" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F9" s="16" t="str">
         <x:v>302b99bbb4073844</x:v>
       </x:c>
@@ -1720,7 +1766,9 @@
       <x:c r="D10" s="16" t="str">
         <x:v>人物走动、滚筒触碰薄膜、中央底座裸露、讲台裸露、双层膜、额外胶带、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E10" s="16" t="str"/>
+      <x:c r="E10" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F10" s="16" t="str">
         <x:v>9c15598cfb500bba</x:v>
       </x:c>
@@ -1738,7 +1786,9 @@
       <x:c r="D11" s="16" t="str">
         <x:v>电视变成平板、屏幕点亮、薄膜穿模、厚机身裸露、双层膜、额外胶带、人物、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E11" s="16" t="str"/>
+      <x:c r="E11" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F11" s="16" t="str">
         <x:v>8b75f65c54dcac7d</x:v>
       </x:c>
@@ -1756,7 +1806,9 @@
       <x:c r="D12" s="16" t="str">
         <x:v>强风掀膜、膜脱落、雨水、胶带松脱、额外胶带、人物靠近、屏幕裸露、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E12" s="16" t="str"/>
+      <x:c r="E12" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>058501105e2b5b9a</x:v>
       </x:c>
@@ -1774,7 +1826,9 @@
       <x:c r="D13" s="16" t="str">
         <x:v>膜贴在电视屏幕上、胶带悬空、壁龛裸露、电视跑到膜前、双层膜、额外胶带、人物触碰、文字、标识、水印</x:v>
       </x:c>
-      <x:c r="E13" s="16" t="str"/>
+      <x:c r="E13" s="16" t="str">
+        <x:v>../../04_电视_墙面固定_完整膜返工/技术记录（不用看）/approved-candidates/电视完整膜基准.png</x:v>
+      </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>51e5b0d1d388fff7</x:v>
       </x:c>
@@ -1785,7 +1839,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f6479f4c0c14f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79cad251e3114cb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1884,13 +1938,27 @@
         <x:v>06_电视_差异化场景/技术记录（不用看）/video-review.json</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="16" t="str">
+        <x:v>扩展七案例案例07</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>学校多媒体教室首帧</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>黄色胶带端点超出透明膜可验证上沿且右端出画，首帧硬门淘汰</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>08_电视_扩展七案例/技术记录（不用看）/keyframe-review.json</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70386a8d0c974529"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R427a2b7c02bf408c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>